<commit_message>
ASN flow 15-Oct: Get Order (X12 on-demand pre-mapping), Hold Flag by D/S, Create ASN mapping, Created status
- X8 prototype: Delivery Date / Rit / Route with Get Order, header Case Qty / PO Readiness / ASN Status,
  two-level D/S expand with Hold / Release, Case List with Delivery Qty and PO detail expand
- X12 becomes the function behind Get Order (temporary #TB_R_INSTRUCTION, no scheduler)
- X10: NSP columns HOLD_FLAG / PO_MAPPED_FLAG kept on re-sync
- X13 reads cases from TB_R_ASN_CROSSDOCK_D; UISS, md and executive overview updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/exec/Crossdock_Executive_Overview.xlsx
+++ b/deliverables/exec/Crossdock_Executive_Overview.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Business Flow" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Executive Summary'!$A$1:$N$29</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Executive Summary'!$A$1:$N$30</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Function Map'!$A$1:$L$20</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Task List'!$A$1:$I$27</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Konfirmasi'!$A$1:$K$31</definedName>
@@ -914,7 +914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:M28"/>
+  <dimension ref="B2:M29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -942,7 +942,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>NSP · disusun oleh FID Rayhan (BSA) · status per 14-Oct-2026</t>
+          <t>NSP · disusun oleh FID Rayhan (BSA) · status per 15-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1127,7 @@
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>X9, X10 replikasi order · X12 order ↔ PO (FIFO) · X8 ASN Crossdock Creation · X13 ASN Inquiry</t>
+          <t>X9, X10 replikasi order · X8 ASN Crossdock Creation (Get Order → X12 pre-mapping, Create ASN, Submit) · X13 ASN Inquiry</t>
         </is>
       </c>
       <c r="E17" s="7" t="n"/>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
-          <t>▸  Update UISS X8 / X13 setelah konfirmasi case label, nomor ASN, route master (FID Rayhan)</t>
+          <t>▸  Update UISS X8 / X13 setelah konfirmasi case label, isi 1 ASN, route master, tabel ASN (FID Rayhan)</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="H22" s="19" t="inlineStr">
         <is>
-          <t>▸  Finalisasi logika FIFO dan struktur Pra Daily Order di UISS X12 (FID Rayhan)</t>
+          <t>▸  Finalisasi struktur Pra Daily Order (mapped qty) di UISS X8 / X12 (FID Rayhan)</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>▸  Konfirmasi struktur tabel Pra Daily Order dan route master (Tim NSP / IT)</t>
+          <t>▸  Tambah kolom HOLD_FLAG / PO_MAPPED_FLAG di H0253 NSP dan cara mempertahankannya saat sync (Tim NSP / IT)</t>
         </is>
       </c>
     </row>
@@ -1224,19 +1224,31 @@
       </c>
       <c r="H26" s="19" t="inlineStr">
         <is>
+          <t>▸  Konfirmasi struktur tabel Pra Daily Order dan route master (Tim NSP / IT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>✔  ASN flow versi 15-Oct: Get Order (X12 on-demand pre-mapping), Hold Flag oleh D/S, Create ASN (mapping), status Ready / Not Ready / Created</t>
+        </is>
+      </c>
+      <c r="H27" s="19" t="inlineStr">
+        <is>
           <t>▸  Susun testing strategy &amp; test scenario (unit, integration, UAT) X1-X13 (FID Rayhan)</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="20" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="20" t="inlineStr">
         <is>
           <t>Detail: sheet Business Flow (alur), Function Map (13 fungsi), Task List, Konfirmasi (keputusan yang dibutuhkan). Prototype: https://ivanrayhannn.github.io/crossdockpoc/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="35">
+  <mergeCells count="37">
     <mergeCell ref="H21:M21"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="D10:E10"/>
@@ -1246,10 +1258,11 @@
     <mergeCell ref="J10:K10"/>
     <mergeCell ref="D15:G15"/>
     <mergeCell ref="H17:M17"/>
+    <mergeCell ref="B29:M29"/>
     <mergeCell ref="H16:M16"/>
     <mergeCell ref="B7:M8"/>
-    <mergeCell ref="B28:M28"/>
     <mergeCell ref="H22:M22"/>
+    <mergeCell ref="H27:M27"/>
     <mergeCell ref="F11:G12"/>
     <mergeCell ref="L11:M12"/>
     <mergeCell ref="B17:C17"/>
@@ -1268,6 +1281,7 @@
     <mergeCell ref="B11:C12"/>
     <mergeCell ref="D11:E12"/>
     <mergeCell ref="D16:G16"/>
+    <mergeCell ref="B27:G27"/>
     <mergeCell ref="H11:I12"/>
     <mergeCell ref="J11:K12"/>
     <mergeCell ref="H25:M25"/>
@@ -1312,7 +1326,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>13 fungsi Crossdock Optimization (UISS X1-X13) · status per 14-Oct-2026</t>
+          <t>13 fungsi Crossdock Optimization (UISS X1-X13) · status per 15-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -1818,12 +1832,12 @@
       </c>
       <c r="H14" s="24" t="inlineStr">
         <is>
-          <t>TB_R_INSTRUCTION</t>
+          <t>Delivery Date, Rit; #TB_R_INSTRUCTION (X12)</t>
         </is>
       </c>
       <c r="I14" s="24" t="inlineStr">
         <is>
-          <t>TB_R_ASN_CROSSDOCK_H, ASN / case no.</t>
+          <t>H0253 flags, TB_R_ASN_CROSSDOCK_H / _D</t>
         </is>
       </c>
       <c r="J14" s="25" t="inlineStr">
@@ -2021,17 +2035,17 @@
       </c>
       <c r="C18" s="24" t="inlineStr">
         <is>
-          <t>Customer Order - PO Mapping</t>
+          <t>Get Order - Customer Order PO Pre-mapping</t>
         </is>
       </c>
       <c r="D18" s="25" t="inlineStr">
         <is>
-          <t>Batch</t>
+          <t>Function</t>
         </is>
       </c>
       <c r="E18" s="24" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Supplier (button in X8)</t>
         </is>
       </c>
       <c r="F18" s="24" t="inlineStr">
@@ -2041,22 +2055,22 @@
       </c>
       <c r="G18" s="24" t="inlineStr">
         <is>
-          <t>Daily (TBC)</t>
+          <t>On demand ([Get Order])</t>
         </is>
       </c>
       <c r="H18" s="24" t="inlineStr">
         <is>
-          <t>H0253 (status 7), Pra Daily Order</t>
+          <t>H0253 (status 7, Hold N), Pra Daily Order</t>
         </is>
       </c>
       <c r="I18" s="24" t="inlineStr">
         <is>
-          <t>TB_R_INSTRUCTION (FIFO by order date)</t>
+          <t>#TB_R_INSTRUCTION (temp, FIFO)</t>
         </is>
       </c>
       <c r="J18" s="25" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Yes (in X8)</t>
         </is>
       </c>
       <c r="K18" s="25" t="inlineStr">
@@ -2103,7 +2117,7 @@
       </c>
       <c r="H19" s="18" t="inlineStr">
         <is>
-          <t>TB_R_ASN_CROSSDOCK_H, TB_R_INSTRUCTION</t>
+          <t>TB_R_ASN_CROSSDOCK_H / _D</t>
         </is>
       </c>
       <c r="I19" s="18" t="inlineStr">
@@ -2164,7 +2178,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Pekerjaan yang masih terbuka per 14-Oct-2026. Kolom Status bisa diubah (pilihan list).</t>
+          <t>Pekerjaan yang masih terbuka per 15-Oct-2026. Kolom Status bisa diubah (pilihan list).</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2292,7 @@
       </c>
       <c r="C13" s="18" t="inlineStr">
         <is>
-          <t>Update UISS X8 / X13 setelah konfirmasi case label, nomor ASN, route master</t>
+          <t>Update UISS X8 / X13 setelah konfirmasi case label, isi 1 ASN, route master, tabel ASN</t>
         </is>
       </c>
       <c r="D13" s="18" t="inlineStr">
@@ -2298,7 +2312,7 @@
       </c>
       <c r="G13" s="18" t="inlineStr">
         <is>
-          <t>Konfirmasi no. 1-8</t>
+          <t>Konfirmasi no. 1-5</t>
         </is>
       </c>
       <c r="H13" s="29" t="inlineStr">
@@ -2318,12 +2332,12 @@
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t>Finalisasi logika FIFO dan struktur Pra Daily Order di UISS X12</t>
+          <t>Finalisasi struktur Pra Daily Order (mapped qty) di UISS X8 / X12</t>
         </is>
       </c>
       <c r="D14" s="18" t="inlineStr">
         <is>
-          <t>X12</t>
+          <t>X8 / X12</t>
         </is>
       </c>
       <c r="E14" s="18" t="inlineStr">
@@ -2358,12 +2372,12 @@
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>Isi jadwal &amp; retry di Schedule sheet UISS X5, X9-X12</t>
+          <t>Isi jadwal &amp; retry di Schedule sheet UISS X5, X9-X11</t>
         </is>
       </c>
       <c r="D15" s="18" t="inlineStr">
         <is>
-          <t>X5, X9-X12</t>
+          <t>X5, X9-X11</t>
         </is>
       </c>
       <c r="E15" s="18" t="inlineStr">
@@ -2558,12 +2572,12 @@
       </c>
       <c r="C20" s="18" t="inlineStr">
         <is>
-          <t>Konfirmasi struktur tabel Pra Daily Order dan route master</t>
+          <t>Tambah kolom HOLD_FLAG / PO_MAPPED_FLAG di H0253 NSP dan cara mempertahankannya saat sync</t>
         </is>
       </c>
       <c r="D20" s="18" t="inlineStr">
         <is>
-          <t>X8, X12</t>
+          <t>X10</t>
         </is>
       </c>
       <c r="E20" s="18" t="inlineStr">
@@ -2578,7 +2592,7 @@
       </c>
       <c r="G20" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Konfirmasi no. 7</t>
         </is>
       </c>
       <c r="H20" s="29" t="inlineStr">
@@ -2598,37 +2612,37 @@
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>Prototype: Download Case Label sesuai format</t>
+          <t>Konfirmasi struktur tabel Pra Daily Order dan route master</t>
         </is>
       </c>
       <c r="D21" s="18" t="inlineStr">
         <is>
-          <t>X8 / X13</t>
+          <t>X8, X12</t>
         </is>
       </c>
       <c r="E21" s="18" t="inlineStr">
         <is>
-          <t>Prototype</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F21" s="18" t="inlineStr">
         <is>
-          <t>FID Rayhan</t>
+          <t>Tim NSP / IT</t>
         </is>
       </c>
       <c r="G21" s="18" t="inlineStr">
         <is>
-          <t>Konfirmasi no. 1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H21" s="29" t="inlineStr">
         <is>
-          <t>Waiting confirmation</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="I21" s="22" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2638,12 +2652,12 @@
       </c>
       <c r="C22" s="18" t="inlineStr">
         <is>
-          <t>Prototype: Case List supplier level case &amp; akses D/S</t>
+          <t>Prototype: Download Case Label sesuai format</t>
         </is>
       </c>
       <c r="D22" s="18" t="inlineStr">
         <is>
-          <t>X8</t>
+          <t>X8 / X13</t>
         </is>
       </c>
       <c r="E22" s="18" t="inlineStr">
@@ -2658,7 +2672,7 @@
       </c>
       <c r="G22" s="18" t="inlineStr">
         <is>
-          <t>Konfirmasi no. 4-5</t>
+          <t>Konfirmasi no. 1</t>
         </is>
       </c>
       <c r="H22" s="29" t="inlineStr">
@@ -2880,7 +2894,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Pertanyaan yang perlu keputusan user per 14-Oct-2026.</t>
+          <t>Pertanyaan yang perlu keputusan user per 15-Oct-2026.</t>
         </is>
       </c>
     </row>
@@ -2997,22 +3011,22 @@
       </c>
       <c r="D9" s="17" t="inlineStr">
         <is>
-          <t>Nomor ASN</t>
+          <t>Isi 1 ASN</t>
         </is>
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>Aturan nomor urut ASN.</t>
+          <t>Apakah 1 ASN wajib 1 supplier / plant?</t>
         </is>
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>ASN-{Supplier}-{YYMMDD Delivery Date}-{Seq 3 digit}, reset per hari per supplier.</t>
+          <t>Ya, 1 ASN = 1 supplier + plant.</t>
         </is>
       </c>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>Format ASN No di X8 / X13 masih usulan.</t>
+          <t>Validasi pilihan unit di Create ASN.</t>
         </is>
       </c>
       <c r="H9" s="30" t="n"/>
@@ -3033,22 +3047,22 @@
       </c>
       <c r="D10" s="17" t="inlineStr">
         <is>
-          <t>Isi 1 ASN</t>
+          <t>Akses D/S</t>
         </is>
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>Apakah 1 ASN wajib 1 supplier / plant?</t>
+          <t>Apakah tim D/S juga boleh Create / Submit ASN, atau hanya melihat + hold?</t>
         </is>
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>Ya, 1 ASN = 1 supplier + plant.</t>
+          <t>Hanya melihat + hold.</t>
         </is>
       </c>
       <c r="G10" s="18" t="inlineStr">
         <is>
-          <t>Validasi pilihan unit di Create ASN.</t>
+          <t>Hak akses tombol Create ASN.</t>
         </is>
       </c>
       <c r="H10" s="30" t="n"/>
@@ -3069,22 +3083,22 @@
       </c>
       <c r="D11" s="17" t="inlineStr">
         <is>
-          <t>Case List supplier</t>
+          <t>Route master</t>
         </is>
       </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>Sub screen Case List untuk supplier juga level case saja (sembunyikan Customer Order No dan pcs)?</t>
+          <t>Nama dan struktur tabel route master (Rit / Route).</t>
         </is>
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>Ya, samakan dengan header (level case).</t>
+          <t>Pakai route master NSP existing.</t>
         </is>
       </c>
       <c r="G11" s="18" t="inlineStr">
         <is>
-          <t>Kolom Case List di UISS X8.</t>
+          <t>Combo Rit masih mock.</t>
         </is>
       </c>
       <c r="H11" s="30" t="n"/>
@@ -3100,27 +3114,27 @@
       </c>
       <c r="C12" s="22" t="inlineStr">
         <is>
-          <t>X8</t>
+          <t>X8 / X13</t>
         </is>
       </c>
       <c r="D12" s="17" t="inlineStr">
         <is>
-          <t>Akses D/S</t>
+          <t>Tabel ASN</t>
         </is>
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>Apakah tim D/S juga boleh Create / Submit ASN, atau hanya melihat?</t>
+          <t>Konfirmasi TB_R_ASN_CROSSDOCK_H / _D (usulan) atau pakai tabel ASN existing.</t>
         </is>
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>Hanya melihat (read only).</t>
+          <t>Pakai usulan di Appendix UISS X8.</t>
         </is>
       </c>
       <c r="G12" s="18" t="inlineStr">
         <is>
-          <t>Hak akses tombol Create ASN.</t>
+          <t>Data mapping Submit ASN.</t>
         </is>
       </c>
       <c r="H12" s="30" t="n"/>
@@ -3141,22 +3155,22 @@
       </c>
       <c r="D13" s="17" t="inlineStr">
         <is>
-          <t>Route master</t>
+          <t>Back / Cancel</t>
         </is>
       </c>
       <c r="E13" s="18" t="inlineStr">
         <is>
-          <t>Nama dan struktur tabel route master (Rit Cycle / Route).</t>
+          <t>Back / Cancel di Case List melepas mapping (PO_MAPPED_FLAG dan qty PO kembali). Setuju?</t>
         </is>
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>Pakai route master NSP existing.</t>
+          <t>Ya.</t>
         </is>
       </c>
       <c r="G13" s="18" t="inlineStr">
         <is>
-          <t>Combo Rit Cycle masih mock.</t>
+          <t>Order bisa terkunci tanpa ASN.</t>
         </is>
       </c>
       <c r="H13" s="30" t="n"/>
@@ -3172,27 +3186,27 @@
       </c>
       <c r="C14" s="22" t="inlineStr">
         <is>
-          <t>X8 / X13</t>
+          <t>X10</t>
         </is>
       </c>
       <c r="D14" s="17" t="inlineStr">
         <is>
-          <t>Tabel header ASN</t>
+          <t>Flag H0253</t>
         </is>
       </c>
       <c r="E14" s="18" t="inlineStr">
         <is>
-          <t>Konfirmasi nama dan kolom TB_R_ASN_CROSSDOCK_H (usulan).</t>
+          <t>HOLD_FLAG dan PO_MAPPED_FLAG dipertahankan per unique key saat delete - insert X10. Setuju?</t>
         </is>
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>Pakai usulan di Appendix UISS X8.</t>
+          <t>Ya (cara teknis oleh tim IT).</t>
         </is>
       </c>
       <c r="G14" s="18" t="inlineStr">
         <is>
-          <t>Data mapping Submit ASN.</t>
+          <t>Hold / mapping hilang setiap sync.</t>
         </is>
       </c>
       <c r="H14" s="30" t="n"/>
@@ -3244,7 +3258,7 @@
       </c>
       <c r="C16" s="22" t="inlineStr">
         <is>
-          <t>X12</t>
+          <t>X8 / X12</t>
         </is>
       </c>
       <c r="D16" s="17" t="inlineStr">
@@ -3254,17 +3268,17 @@
       </c>
       <c r="E16" s="18" t="inlineStr">
         <is>
-          <t>Struktur fisik TB_R_PRA_DAILY_ORDER_MANIFEST / PART dan cara menandai PO yang sudah terpasang.</t>
+          <t>Struktur fisik TB_R_PRA_DAILY_ORDER_MANIFEST / PART dan kolom qty terpakai (mapped qty).</t>
         </is>
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>Tambah flag / qty terpakai di PART.</t>
+          <t>Tambah kolom MAPPED_QTY di PART.</t>
         </is>
       </c>
       <c r="G16" s="18" t="inlineStr">
         <is>
-          <t>Logika FIFO X12 belum final.</t>
+          <t>Logika FIFO X12 / Create ASN belum final.</t>
         </is>
       </c>
       <c r="H16" s="30" t="n"/>
@@ -3280,7 +3294,7 @@
       </c>
       <c r="C17" s="22" t="inlineStr">
         <is>
-          <t>X9-X12</t>
+          <t>X9-X11</t>
         </is>
       </c>
       <c r="D17" s="17" t="inlineStr">
@@ -3290,7 +3304,7 @@
       </c>
       <c r="E17" s="18" t="inlineStr">
         <is>
-          <t>Jadwal scheduler NSP untuk X9, X10, X11, X12 dan perlu auto retry seperti X6 / X7?</t>
+          <t>Jadwal scheduler NSP untuk X9, X10, X11 dan perlu auto retry seperti X6 / X7?</t>
         </is>
       </c>
       <c r="F17" s="18" t="inlineStr">
@@ -4328,30 +4342,7 @@
       </c>
       <c r="AB14" s="46" t="n"/>
       <c r="AC14" s="46" t="n"/>
-      <c r="AD14" s="47" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00C00000"/>
-              <sz val="9"/>
-            </rPr>
-            <t xml:space="preserve">X12
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00262626"/>
-              <sz val="9"/>
-            </rPr>
-            <t>Customer order ↔ PO
-mapping (FIFO by
-order date)</t>
-          </r>
-        </is>
-      </c>
+      <c r="AD14" s="46" t="n"/>
       <c r="AE14" s="46" t="n"/>
       <c r="AF14" s="46" t="n"/>
       <c r="AG14" s="46" t="n"/>
@@ -4406,13 +4397,9 @@
       </c>
       <c r="AA15" s="49" t="n"/>
       <c r="AB15" s="40" t="n"/>
-      <c r="AC15" s="48" t="inlineStr">
-        <is>
-          <t>►</t>
-        </is>
-      </c>
-      <c r="AD15" s="49" t="n"/>
-      <c r="AE15" s="40" t="n"/>
+      <c r="AC15" s="46" t="n"/>
+      <c r="AD15" s="46" t="n"/>
+      <c r="AE15" s="46" t="n"/>
       <c r="AF15" s="46" t="n"/>
       <c r="AG15" s="46" t="n"/>
       <c r="AH15" s="46" t="n"/>
@@ -4449,10 +4436,10 @@
       <c r="Y16" s="46" t="n"/>
       <c r="Z16" s="46" t="n"/>
       <c r="AA16" s="50" t="n"/>
-      <c r="AB16" s="46" t="n"/>
+      <c r="AB16" s="40" t="n"/>
       <c r="AC16" s="46" t="n"/>
-      <c r="AD16" s="50" t="n"/>
-      <c r="AE16" s="40" t="n"/>
+      <c r="AD16" s="46" t="n"/>
+      <c r="AE16" s="46" t="n"/>
       <c r="AF16" s="46" t="n"/>
       <c r="AG16" s="46" t="n"/>
       <c r="AH16" s="46" t="n"/>
@@ -4489,10 +4476,10 @@
       <c r="Y17" s="51" t="n"/>
       <c r="Z17" s="51" t="n"/>
       <c r="AA17" s="51" t="n"/>
-      <c r="AB17" s="51" t="n"/>
+      <c r="AB17" s="44" t="n"/>
       <c r="AC17" s="51" t="n"/>
       <c r="AD17" s="51" t="n"/>
-      <c r="AE17" s="44" t="n"/>
+      <c r="AE17" s="51" t="n"/>
       <c r="AF17" s="51" t="n"/>
       <c r="AG17" s="51" t="n"/>
       <c r="AH17" s="51" t="n"/>
@@ -4533,10 +4520,10 @@
       <c r="Y18" s="35" t="n"/>
       <c r="Z18" s="35" t="n"/>
       <c r="AA18" s="35" t="n"/>
-      <c r="AB18" s="35" t="n"/>
+      <c r="AB18" s="40" t="n"/>
       <c r="AC18" s="35" t="n"/>
       <c r="AD18" s="35" t="n"/>
-      <c r="AE18" s="40" t="n"/>
+      <c r="AE18" s="35" t="n"/>
       <c r="AF18" s="35" t="n"/>
       <c r="AG18" s="35" t="n"/>
       <c r="AH18" s="35" t="n"/>
@@ -4596,10 +4583,10 @@
       <c r="Y19" s="35" t="n"/>
       <c r="Z19" s="35" t="n"/>
       <c r="AA19" s="35" t="n"/>
-      <c r="AB19" s="35" t="n"/>
+      <c r="AB19" s="40" t="n"/>
       <c r="AC19" s="35" t="n"/>
       <c r="AD19" s="35" t="n"/>
-      <c r="AE19" s="40" t="n"/>
+      <c r="AE19" s="35" t="n"/>
       <c r="AF19" s="35" t="n"/>
       <c r="AG19" s="35" t="n"/>
       <c r="AH19" s="35" t="n"/>
@@ -4636,10 +4623,10 @@
       <c r="Y20" s="35" t="n"/>
       <c r="Z20" s="35" t="n"/>
       <c r="AA20" s="35" t="n"/>
-      <c r="AB20" s="35" t="n"/>
+      <c r="AB20" s="40" t="n"/>
       <c r="AC20" s="35" t="n"/>
       <c r="AD20" s="35" t="n"/>
-      <c r="AE20" s="40" t="n"/>
+      <c r="AE20" s="35" t="n"/>
       <c r="AF20" s="35" t="n"/>
       <c r="AG20" s="35" t="n"/>
       <c r="AH20" s="35" t="n"/>
@@ -4676,10 +4663,10 @@
       <c r="Y21" s="35" t="n"/>
       <c r="Z21" s="35" t="n"/>
       <c r="AA21" s="35" t="n"/>
-      <c r="AB21" s="35" t="n"/>
+      <c r="AB21" s="40" t="n"/>
       <c r="AC21" s="35" t="n"/>
       <c r="AD21" s="35" t="n"/>
-      <c r="AE21" s="40" t="n"/>
+      <c r="AE21" s="35" t="n"/>
       <c r="AF21" s="35" t="n"/>
       <c r="AG21" s="35" t="n"/>
       <c r="AH21" s="35" t="n"/>
@@ -4716,10 +4703,10 @@
       <c r="Y22" s="43" t="n"/>
       <c r="Z22" s="43" t="n"/>
       <c r="AA22" s="43" t="n"/>
-      <c r="AB22" s="43" t="n"/>
+      <c r="AB22" s="44" t="n"/>
       <c r="AC22" s="43" t="n"/>
       <c r="AD22" s="43" t="n"/>
-      <c r="AE22" s="44" t="n"/>
+      <c r="AE22" s="43" t="n"/>
       <c r="AF22" s="43" t="n"/>
       <c r="AG22" s="43" t="n"/>
       <c r="AH22" s="43" t="n"/>
@@ -4760,10 +4747,10 @@
       <c r="Y23" s="46" t="n"/>
       <c r="Z23" s="46" t="n"/>
       <c r="AA23" s="46" t="n"/>
-      <c r="AB23" s="46" t="n"/>
+      <c r="AB23" s="40" t="n"/>
       <c r="AC23" s="46" t="n"/>
       <c r="AD23" s="46" t="n"/>
-      <c r="AE23" s="40" t="n"/>
+      <c r="AE23" s="46" t="n"/>
       <c r="AF23" s="46" t="n"/>
       <c r="AG23" s="46" t="n"/>
       <c r="AH23" s="46" t="n"/>
@@ -4823,12 +4810,9 @@
       <c r="Y24" s="46" t="n"/>
       <c r="Z24" s="46" t="n"/>
       <c r="AA24" s="46" t="n"/>
-      <c r="AB24" s="46" t="n"/>
+      <c r="AB24" s="40" t="n"/>
       <c r="AC24" s="46" t="n"/>
-      <c r="AD24" s="46" t="n"/>
-      <c r="AE24" s="40" t="n"/>
-      <c r="AF24" s="46" t="n"/>
-      <c r="AG24" s="57" t="inlineStr">
+      <c r="AD24" s="57" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4846,11 +4830,14 @@
               <color rgb="00262626"/>
               <sz val="9"/>
             </rPr>
-            <t>Monitor delivery plan
-(destination, pcs)</t>
+            <t>Monitor detail &amp;
+hold order line</t>
           </r>
         </is>
       </c>
+      <c r="AE24" s="46" t="n"/>
+      <c r="AF24" s="46" t="n"/>
+      <c r="AG24" s="46" t="n"/>
       <c r="AH24" s="46" t="n"/>
       <c r="AI24" s="46" t="n"/>
       <c r="AJ24" s="46" t="n"/>
@@ -4889,16 +4876,16 @@
       <c r="Y25" s="46" t="n"/>
       <c r="Z25" s="46" t="n"/>
       <c r="AA25" s="46" t="n"/>
-      <c r="AB25" s="46" t="n"/>
-      <c r="AC25" s="46" t="n"/>
-      <c r="AD25" s="46" t="n"/>
+      <c r="AB25" s="40" t="n"/>
+      <c r="AC25" s="48" t="inlineStr">
+        <is>
+          <t>►</t>
+        </is>
+      </c>
+      <c r="AD25" s="58" t="n"/>
       <c r="AE25" s="40" t="n"/>
-      <c r="AF25" s="48" t="inlineStr">
-        <is>
-          <t>►</t>
-        </is>
-      </c>
-      <c r="AG25" s="58" t="n"/>
+      <c r="AF25" s="46" t="n"/>
+      <c r="AG25" s="46" t="n"/>
       <c r="AH25" s="46" t="n"/>
       <c r="AI25" s="46" t="n"/>
       <c r="AJ25" s="46" t="n"/>
@@ -4933,12 +4920,12 @@
       <c r="Y26" s="46" t="n"/>
       <c r="Z26" s="46" t="n"/>
       <c r="AA26" s="46" t="n"/>
-      <c r="AB26" s="46" t="n"/>
+      <c r="AB26" s="40" t="n"/>
       <c r="AC26" s="46" t="n"/>
-      <c r="AD26" s="46" t="n"/>
+      <c r="AD26" s="59" t="n"/>
       <c r="AE26" s="40" t="n"/>
       <c r="AF26" s="46" t="n"/>
-      <c r="AG26" s="59" t="n"/>
+      <c r="AG26" s="46" t="n"/>
       <c r="AH26" s="46" t="n"/>
       <c r="AI26" s="46" t="n"/>
       <c r="AJ26" s="46" t="n"/>
@@ -4973,7 +4960,7 @@
       <c r="Y27" s="51" t="n"/>
       <c r="Z27" s="51" t="n"/>
       <c r="AA27" s="51" t="n"/>
-      <c r="AB27" s="51" t="n"/>
+      <c r="AB27" s="44" t="n"/>
       <c r="AC27" s="51" t="n"/>
       <c r="AD27" s="51" t="n"/>
       <c r="AE27" s="44" t="n"/>
@@ -5017,7 +5004,7 @@
       <c r="Y28" s="35" t="n"/>
       <c r="Z28" s="35" t="n"/>
       <c r="AA28" s="35" t="n"/>
-      <c r="AB28" s="35" t="n"/>
+      <c r="AB28" s="40" t="n"/>
       <c r="AC28" s="35" t="n"/>
       <c r="AD28" s="35" t="n"/>
       <c r="AE28" s="40" t="n"/>
@@ -5057,9 +5044,32 @@
       <c r="Y29" s="35" t="n"/>
       <c r="Z29" s="35" t="n"/>
       <c r="AA29" s="35" t="n"/>
-      <c r="AB29" s="35" t="n"/>
+      <c r="AB29" s="40" t="n"/>
       <c r="AC29" s="35" t="n"/>
-      <c r="AD29" s="35" t="n"/>
+      <c r="AD29" s="61" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00C00000"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">X8 → X12
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00262626"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Get Order: order ↔ PO
+pre-mapping (FIFO)
+→ Ready / Not Ready</t>
+          </r>
+        </is>
+      </c>
       <c r="AE29" s="40" t="n"/>
       <c r="AF29" s="35" t="n"/>
       <c r="AG29" s="61" t="inlineStr">
@@ -5080,9 +5090,9 @@
               <color rgb="00262626"/>
               <sz val="9"/>
             </rPr>
-            <t>ASN Crossdock Creation:
-ready units → cases
-→ Submit ASN</t>
+            <t>Create ASN (mapping)
+→ Case List
+→ Submit (Created)</t>
           </r>
         </is>
       </c>
@@ -5165,9 +5175,13 @@
       <c r="Y30" s="35" t="n"/>
       <c r="Z30" s="35" t="n"/>
       <c r="AA30" s="35" t="n"/>
-      <c r="AB30" s="35" t="n"/>
-      <c r="AC30" s="35" t="n"/>
-      <c r="AD30" s="35" t="n"/>
+      <c r="AB30" s="40" t="n"/>
+      <c r="AC30" s="63" t="inlineStr">
+        <is>
+          <t>►</t>
+        </is>
+      </c>
+      <c r="AD30" s="64" t="n"/>
       <c r="AE30" s="40" t="n"/>
       <c r="AF30" s="63" t="inlineStr">
         <is>
@@ -5219,7 +5233,7 @@
       <c r="AA31" s="35" t="n"/>
       <c r="AB31" s="35" t="n"/>
       <c r="AC31" s="35" t="n"/>
-      <c r="AD31" s="35" t="n"/>
+      <c r="AD31" s="66" t="n"/>
       <c r="AE31" s="35" t="n"/>
       <c r="AF31" s="35" t="n"/>
       <c r="AG31" s="66" t="n"/>
@@ -5540,7 +5554,7 @@
       </c>
       <c r="X43" s="74" t="inlineStr">
         <is>
-          <t>2.  Order dipasangkan ke PO supplier secara FIFO berdasarkan order date.</t>
+          <t>2.  Get Order: order dipasangkan ke PO secara FIFO (pre-mapping); mapping final saat Create ASN.</t>
         </is>
       </c>
     </row>
@@ -5564,7 +5578,7 @@
       </c>
       <c r="X45" s="74" t="inlineStr">
         <is>
-          <t>4.  Supplier melihat level case; detail destinasi &amp; pcs hanya untuk D/S team.</t>
+          <t>4.  Supplier melihat level case; detail &amp; Hold Flag order line hanya untuk D/S team.</t>
         </is>
       </c>
     </row>
@@ -5614,7 +5628,6 @@
     <mergeCell ref="B28:B32"/>
     <mergeCell ref="I14:I16"/>
     <mergeCell ref="AJ29:AJ31"/>
-    <mergeCell ref="AG24:AG26"/>
     <mergeCell ref="F14:F16"/>
     <mergeCell ref="X9:X11"/>
     <mergeCell ref="X44:AM44"/>
@@ -5624,10 +5637,11 @@
     <mergeCell ref="X43:AM43"/>
     <mergeCell ref="AA14:AA16"/>
     <mergeCell ref="F19:F21"/>
+    <mergeCell ref="AD24:AD26"/>
     <mergeCell ref="C6:R6"/>
     <mergeCell ref="C42:R42"/>
-    <mergeCell ref="AD14:AD16"/>
     <mergeCell ref="C45:R45"/>
+    <mergeCell ref="AD29:AD31"/>
     <mergeCell ref="O24:O26"/>
     <mergeCell ref="R34:R36"/>
     <mergeCell ref="AM29:AM31"/>

</xml_diff>

<commit_message>
ASN Crossdock Creation: Search button, default delivery date today, hide readiness 0 and Created units, destination-level Hold Flag
- D/S detail is destination level only (Destination, Case, Qty, Hold Flag); customer order lines,
  Assignment and Not Assigned (pcs) removed
- X8 / X12 UISS and md, executive overview updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/exec/Crossdock_Executive_Overview.xlsx
+++ b/deliverables/exec/Crossdock_Executive_Overview.xlsx
@@ -1127,7 +1127,7 @@
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>X9, X10 replikasi order · X8 ASN Crossdock Creation (Get Order → X12 pre-mapping, Create ASN, Submit) · X13 ASN Inquiry</t>
+          <t>X9, X10 replikasi order · X8 ASN Crossdock Creation (Search → X12 pre-mapping, Create ASN, Submit) · X13 ASN Inquiry</t>
         </is>
       </c>
       <c r="E17" s="7" t="n"/>
@@ -1231,7 +1231,7 @@
     <row r="27" ht="30" customHeight="1">
       <c r="B27" s="19" t="inlineStr">
         <is>
-          <t>✔  ASN flow versi 15-Oct: Get Order (X12 on-demand pre-mapping), Hold Flag oleh D/S, Create ASN (mapping), status Ready / Not Ready / Created</t>
+          <t>✔  ASN flow versi 15-Oct: Search (X12 on-demand pre-mapping), Hold Flag per destinasi oleh D/S, Create ASN (mapping), status Ready / Not Ready / Created</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="G18" s="24" t="inlineStr">
         <is>
-          <t>On demand ([Get Order])</t>
+          <t>On demand ([Search] in X8)</t>
         </is>
       </c>
       <c r="H18" s="24" t="inlineStr">
@@ -4831,7 +4831,7 @@
               <sz val="9"/>
             </rPr>
             <t>Monitor detail &amp;
-hold order line</t>
+hold destination</t>
           </r>
         </is>
       </c>
@@ -5064,8 +5064,8 @@
               <color rgb="00262626"/>
               <sz val="9"/>
             </rPr>
-            <t>Get Order: order ↔ PO
-pre-mapping (FIFO)
+            <t>Search (Get Order):
+order ↔ PO pre-mapping
 → Ready / Not Ready</t>
           </r>
         </is>
@@ -5554,7 +5554,7 @@
       </c>
       <c r="X43" s="74" t="inlineStr">
         <is>
-          <t>2.  Get Order: order dipasangkan ke PO secara FIFO (pre-mapping); mapping final saat Create ASN.</t>
+          <t>2.  Search: order dipasangkan ke PO secara FIFO (pre-mapping); mapping final saat Create ASN.</t>
         </is>
       </c>
     </row>
@@ -5578,7 +5578,7 @@
       </c>
       <c r="X45" s="74" t="inlineStr">
         <is>
-          <t>4.  Supplier melihat level case; detail &amp; Hold Flag order line hanya untuk D/S team.</t>
+          <t>4.  Supplier melihat level case; detail &amp; Hold Flag destinasi hanya untuk D/S team.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Menu Settings admin panel, ASN submit as batch X14 with Submit ID and log, hold check on Create ASN, ASN Backend Process page
- Sidebar menus can be shown / hidden in Common > Menu Settings (kept in the browser)
- Submit ASN hands the draft to batch X14 with a Submit ID; the success message goes to Log Monitoring
- Create ASN re-checks the ticked units: a hold by the D/S team in another session fails the create
  with 'Some order has been already hold, please select other records' and refreshes the selection
- Each View as keeps its own selection to simulate two sessions
- New UISS X14 ASN Submit; X8 / X13 UISS and md, executive overview updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/exec/Crossdock_Executive_Overview.xlsx
+++ b/deliverables/exec/Crossdock_Executive_Overview.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Business Flow" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Executive Summary'!$A$1:$N$30</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Function Map'!$A$1:$L$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Executive Summary'!$A$1:$N$31</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Function Map'!$A$1:$L$21</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Task List'!$A$1:$I$27</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Konfirmasi'!$A$1:$K$31</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'Business Flow'!$A$1:$AN$52</definedName>
@@ -914,7 +914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:M29"/>
+  <dimension ref="B2:M30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1015,17 +1015,17 @@
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="B11" s="10">
-        <f>COUNTA('Function Map'!$B$7:$B$19)</f>
+        <f>COUNTA('Function Map'!$B$7:$B$20)</f>
         <v/>
       </c>
       <c r="C11" s="11" t="n"/>
       <c r="D11" s="10">
-        <f>COUNTIF('Function Map'!$D$7:$D$19,"Screen")</f>
+        <f>COUNTIF('Function Map'!$D$7:$D$20,"Screen")</f>
         <v/>
       </c>
       <c r="E11" s="11" t="n"/>
       <c r="F11" s="10">
-        <f>COUNTIF('Function Map'!$D$7:$D$19,"Batch")</f>
+        <f>COUNTIF('Function Map'!$D$7:$D$20,"Batch")</f>
         <v/>
       </c>
       <c r="G11" s="11" t="n"/>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="K11" s="11" t="n"/>
       <c r="L11" s="13">
-        <f>COUNTIFS('Function Map'!$D$7:$D$19,"Screen",'Function Map'!$J$7:$J$19,"Yes")</f>
+        <f>COUNTIFS('Function Map'!$D$7:$D$20,"Screen",'Function Map'!$J$7:$J$20,"Yes")</f>
         <v/>
       </c>
       <c r="M11" s="11" t="n"/>
@@ -1127,7 +1127,7 @@
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>X9, X10 replikasi order · X8 ASN Crossdock Creation (Search → X12 pre-mapping, Create ASN, Submit) · X13 ASN Inquiry</t>
+          <t>X9, X10 replikasi order · X8 ASN Crossdock Creation (Search → X12 pre-mapping, Create ASN, Submit → X14 batch) · X13 ASN Inquiry</t>
         </is>
       </c>
       <c r="E17" s="7" t="n"/>
@@ -1159,7 +1159,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="B21" s="19" t="inlineStr">
         <is>
-          <t>✔  UISS 13 fungsi (X1-X13) versi 0.1 + file .md per fungsi</t>
+          <t>✔  UISS 14 fungsi (X1-X14) versi 0.1 + file .md per fungsi</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>▸  Review UISS X1-X13 versi 0.1 oleh user / reviewer (User)</t>
+          <t>▸  Review UISS X1-X14 versi 0.1 oleh user / reviewer (User)</t>
         </is>
       </c>
     </row>
@@ -1236,19 +1236,26 @@
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>▸  Susun testing strategy &amp; test scenario (unit, integration, UAT) X1-X13 (FID Rayhan)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="20" t="inlineStr">
-        <is>
-          <t>Detail: sheet Business Flow (alur), Function Map (13 fungsi), Task List, Konfirmasi (keputusan yang dibutuhkan). Prototype: https://ivanrayhannn.github.io/crossdockpoc/</t>
+          <t>▸  Susun testing strategy &amp; test scenario (unit, integration, UAT) X1-X14 (FID Rayhan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>✔  Submit ASN sebagai batch X14 (Submit ID, hasil ke log), cek hold saat Create ASN, admin panel Menu Settings, menu ASN Backend Process</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="20" t="inlineStr">
+        <is>
+          <t>Detail: sheet Business Flow (alur), Function Map (X1-X14), Task List, Konfirmasi (keputusan yang dibutuhkan). Prototype: https://ivanrayhannn.github.io/crossdockpoc/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="37">
+  <mergeCells count="38">
     <mergeCell ref="H21:M21"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="D10:E10"/>
@@ -1258,14 +1265,15 @@
     <mergeCell ref="J10:K10"/>
     <mergeCell ref="D15:G15"/>
     <mergeCell ref="H17:M17"/>
-    <mergeCell ref="B29:M29"/>
     <mergeCell ref="H16:M16"/>
     <mergeCell ref="B7:M8"/>
+    <mergeCell ref="B28:G28"/>
     <mergeCell ref="H22:M22"/>
     <mergeCell ref="H27:M27"/>
     <mergeCell ref="F11:G12"/>
     <mergeCell ref="L11:M12"/>
     <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B30:M30"/>
     <mergeCell ref="B24:G24"/>
     <mergeCell ref="H15:M15"/>
     <mergeCell ref="H24:M24"/>
@@ -1299,7 +1307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:L19"/>
+  <dimension ref="B2:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1326,7 +1334,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>13 fungsi Crossdock Optimization (UISS X1-X13) · status per 15-Oct-2026</t>
+          <t>14 fungsi Crossdock Optimization (UISS X1-X14) · status per 15-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -1837,7 +1845,7 @@
       </c>
       <c r="I14" s="24" t="inlineStr">
         <is>
-          <t>H0253 flags, TB_R_ASN_CROSSDOCK_H / _D</t>
+          <t>H0253 flags, #TEMP_ASN_DRAFT, Submit ID to X14</t>
         </is>
       </c>
       <c r="J14" s="25" t="inlineStr">
@@ -2136,6 +2144,63 @@
         </is>
       </c>
       <c r="L19" s="22" t="inlineStr">
+        <is>
+          <t>Updated</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>X14</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="inlineStr">
+        <is>
+          <t>ASN Submit</t>
+        </is>
+      </c>
+      <c r="D20" s="25" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="E20" s="24" t="inlineStr">
+        <is>
+          <t>System ([Submit ASN] in X8)</t>
+        </is>
+      </c>
+      <c r="F20" s="24" t="inlineStr">
+        <is>
+          <t>B. Daily operation</t>
+        </is>
+      </c>
+      <c r="G20" s="24" t="inlineStr">
+        <is>
+          <t>On demand (Submit ID)</t>
+        </is>
+      </c>
+      <c r="H20" s="24" t="inlineStr">
+        <is>
+          <t>#TEMP_ASN_DRAFT, Submit ID</t>
+        </is>
+      </c>
+      <c r="I20" s="24" t="inlineStr">
+        <is>
+          <t>TB_R_ASN_CROSSDOCK_H / _D, log (existing)</t>
+        </is>
+      </c>
+      <c r="J20" s="25" t="inlineStr">
+        <is>
+          <t>Yes (in X8 + Log Monitoring)</t>
+        </is>
+      </c>
+      <c r="K20" s="25" t="inlineStr">
+        <is>
+          <t>Draft 0.1</t>
+        </is>
+      </c>
+      <c r="L20" s="25" t="inlineStr">
         <is>
           <t>Updated</t>
         </is>
@@ -2457,7 +2522,7 @@
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>X1-X13</t>
+          <t>X1-X14</t>
         </is>
       </c>
       <c r="E17" s="18" t="inlineStr">
@@ -2492,12 +2557,12 @@
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>Review UISS X1-X13 versi 0.1 oleh user / reviewer</t>
+          <t>Review UISS X1-X14 versi 0.1 oleh user / reviewer</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
         <is>
-          <t>X1-X13</t>
+          <t>X1-X14</t>
         </is>
       </c>
       <c r="E18" s="18" t="inlineStr">
@@ -2732,12 +2797,12 @@
       </c>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>Susun testing strategy &amp; test scenario (unit, integration, UAT) X1-X13</t>
+          <t>Susun testing strategy &amp; test scenario (unit, integration, UAT) X1-X14</t>
         </is>
       </c>
       <c r="D24" s="18" t="inlineStr">
         <is>
-          <t>X1-X13</t>
+          <t>X1-X14</t>
         </is>
       </c>
       <c r="E24" s="18" t="inlineStr">
@@ -5081,7 +5146,7 @@
               <color rgb="00C00000"/>
               <sz val="9"/>
             </rPr>
-            <t xml:space="preserve">X8
+            <t xml:space="preserve">X8 → X14
 </t>
           </r>
           <r>
@@ -5091,8 +5156,8 @@
               <sz val="9"/>
             </rPr>
             <t>Create ASN (mapping)
-→ Case List
-→ Submit (Created)</t>
+→ Case List → Submit
+(batch, Submit ID)</t>
           </r>
         </is>
       </c>
@@ -5593,7 +5658,7 @@
       <c r="B48" s="75" t="n"/>
       <c r="C48" s="76" t="inlineStr">
         <is>
-          <t>Kotak = langkah / fungsi; kode merah = UISS (X1-X13)</t>
+          <t>Kotak = langkah / fungsi; kode merah = UISS (X1-X14)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: MSG8 text with automatic refresh, new UISS / md X15 Menu Settings, task list and executive overview
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/exec/Crossdock_Executive_Overview.xlsx
+++ b/deliverables/exec/Crossdock_Executive_Overview.xlsx
@@ -15,9 +15,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Executive Summary'!$A$1:$N$31</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Function Map'!$A$1:$L$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Function Map'!$A$1:$L$22</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Task List'!$A$1:$I$27</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Konfirmasi'!$A$1:$K$31</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Konfirmasi'!$A$1:$K$32</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'Business Flow'!$A$1:$AN$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1015,17 +1015,17 @@
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="B11" s="10">
-        <f>COUNTA('Function Map'!$B$7:$B$20)</f>
+        <f>COUNTA('Function Map'!$B$7:$B$21)</f>
         <v/>
       </c>
       <c r="C11" s="11" t="n"/>
       <c r="D11" s="10">
-        <f>COUNTIF('Function Map'!$D$7:$D$20,"Screen")</f>
+        <f>COUNTIF('Function Map'!$D$7:$D$21,"Screen")</f>
         <v/>
       </c>
       <c r="E11" s="11" t="n"/>
       <c r="F11" s="10">
-        <f>COUNTIF('Function Map'!$D$7:$D$20,"Batch")</f>
+        <f>COUNTIF('Function Map'!$D$7:$D$21,"Batch")</f>
         <v/>
       </c>
       <c r="G11" s="11" t="n"/>
@@ -1035,12 +1035,12 @@
       </c>
       <c r="I11" s="11" t="n"/>
       <c r="J11" s="12">
-        <f>COUNTIF(Konfirmasi!$J$8:$J$30,"Open")</f>
+        <f>COUNTIF(Konfirmasi!$J$8:$J$31,"Open")</f>
         <v/>
       </c>
       <c r="K11" s="11" t="n"/>
       <c r="L11" s="13">
-        <f>COUNTIFS('Function Map'!$D$7:$D$20,"Screen",'Function Map'!$J$7:$J$20,"Yes")</f>
+        <f>COUNTIFS('Function Map'!$D$7:$D$21,"Screen",'Function Map'!$J$7:$J$21,"Yes")</f>
         <v/>
       </c>
       <c r="M11" s="11" t="n"/>
@@ -1159,7 +1159,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="B21" s="19" t="inlineStr">
         <is>
-          <t>✔  UISS 14 fungsi (X1-X14) versi 0.1 + file .md per fungsi</t>
+          <t>✔  UISS 15 fungsi (X1-X15) versi 0.1 + file .md per fungsi</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>▸  Review UISS X1-X14 versi 0.1 oleh user / reviewer (User)</t>
+          <t>▸  Review UISS X1-X15 versi 0.1 oleh user / reviewer (User)</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>▸  Susun testing strategy &amp; test scenario (unit, integration, UAT) X1-X14 (FID Rayhan)</t>
+          <t>▸  Susun testing strategy &amp; test scenario (unit, integration, UAT) X1-X15 (FID Rayhan)</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1250,7 @@
     <row r="30">
       <c r="B30" s="20" t="inlineStr">
         <is>
-          <t>Detail: sheet Business Flow (alur), Function Map (X1-X14), Task List, Konfirmasi (keputusan yang dibutuhkan). Prototype: https://ivanrayhannn.github.io/crossdockpoc/</t>
+          <t>Detail: sheet Business Flow (alur), Function Map (X1-X15), Task List, Konfirmasi (keputusan yang dibutuhkan). Prototype: https://ivanrayhannn.github.io/crossdockpoc/</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:L20"/>
+  <dimension ref="B2:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1334,7 +1334,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>14 fungsi Crossdock Optimization (UISS X1-X14) · status per 15-Oct-2026</t>
+          <t>15 fungsi Crossdock Optimization (UISS X1-X15) · status per 15-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -2201,6 +2201,63 @@
         </is>
       </c>
       <c r="L20" s="25" t="inlineStr">
+        <is>
+          <t>Updated</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>X15</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Menu Settings (admin panel)</t>
+        </is>
+      </c>
+      <c r="D21" s="22" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="G21" s="18" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="H21" s="18" t="inlineStr">
+        <is>
+          <t>Sidebar menu list</t>
+        </is>
+      </c>
+      <c r="I21" s="18" t="inlineStr">
+        <is>
+          <t>TB_M_MENU_VISIBILITY (show / hide)</t>
+        </is>
+      </c>
+      <c r="J21" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K21" s="22" t="inlineStr">
+        <is>
+          <t>Draft 0.1</t>
+        </is>
+      </c>
+      <c r="L21" s="22" t="inlineStr">
         <is>
           <t>Updated</t>
         </is>
@@ -2522,7 +2579,7 @@
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>X1-X14</t>
+          <t>X1-X15</t>
         </is>
       </c>
       <c r="E17" s="18" t="inlineStr">
@@ -2557,12 +2614,12 @@
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>Review UISS X1-X14 versi 0.1 oleh user / reviewer</t>
+          <t>Review UISS X1-X15 versi 0.1 oleh user / reviewer</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
         <is>
-          <t>X1-X14</t>
+          <t>X1-X15</t>
         </is>
       </c>
       <c r="E18" s="18" t="inlineStr">
@@ -2797,12 +2854,12 @@
       </c>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>Susun testing strategy &amp; test scenario (unit, integration, UAT) X1-X14</t>
+          <t>Susun testing strategy &amp; test scenario (unit, integration, UAT) X1-X15</t>
         </is>
       </c>
       <c r="D24" s="18" t="inlineStr">
         <is>
-          <t>X1-X14</t>
+          <t>X1-X15</t>
         </is>
       </c>
       <c r="E24" s="18" t="inlineStr">
@@ -2934,7 +2991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K30"/>
+  <dimension ref="B2:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -3827,27 +3884,27 @@
       </c>
       <c r="C30" s="22" t="inlineStr">
         <is>
-          <t>X1</t>
+          <t>X15</t>
         </is>
       </c>
       <c r="D30" s="17" t="inlineStr">
         <is>
-          <t>Effective Start Date</t>
+          <t>Menu Settings</t>
         </is>
       </c>
       <c r="E30" s="18" t="inlineStr">
         <is>
-          <t>Kalimat "Effective Start Date" yang menggantung di Op Desc 5.4 a.4 (UISS X1): aturan apa yang dimaksud?</t>
+          <t>Pengaturan show / hide menu berlaku per role atau global, dan siapa yang boleh membuka layar ini?</t>
         </is>
       </c>
       <c r="F30" s="18" t="inlineStr">
         <is>
-          <t>Default besok, minimum hari ini, wajib diisi.</t>
+          <t>Per role; hanya admin.</t>
         </is>
       </c>
       <c r="G30" s="18" t="inlineStr">
         <is>
-          <t>Op Desc X1 belum lengkap.</t>
+          <t>Struktur TB_M_MENU_VISIBILITY.</t>
         </is>
       </c>
       <c r="H30" s="30" t="n"/>
@@ -3857,8 +3914,44 @@
         <v/>
       </c>
     </row>
+    <row r="31" ht="42" customHeight="1">
+      <c r="B31" s="22" t="n">
+        <v>24</v>
+      </c>
+      <c r="C31" s="22" t="inlineStr">
+        <is>
+          <t>X1</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>Effective Start Date</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="inlineStr">
+        <is>
+          <t>Kalimat "Effective Start Date" yang menggantung di Op Desc 5.4 a.4 (UISS X1): aturan apa yang dimaksud?</t>
+        </is>
+      </c>
+      <c r="F31" s="18" t="inlineStr">
+        <is>
+          <t>Default besok, minimum hari ini, wajib diisi.</t>
+        </is>
+      </c>
+      <c r="G31" s="18" t="inlineStr">
+        <is>
+          <t>Op Desc X1 belum lengkap.</t>
+        </is>
+      </c>
+      <c r="H31" s="30" t="n"/>
+      <c r="I31" s="30" t="n"/>
+      <c r="J31" s="31">
+        <f>IF(H31="","Open","Decided")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="J8:J30">
+  <conditionalFormatting sqref="J8:J31">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Open"</formula>
     </cfRule>
@@ -5658,7 +5751,7 @@
       <c r="B48" s="75" t="n"/>
       <c r="C48" s="76" t="inlineStr">
         <is>
-          <t>Kotak = langkah / fungsi; kode merah = UISS (X1-X14)</t>
+          <t>Kotak = langkah / fungsi; kode merah = UISS (X1-X15)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ASN: apply confirmations 1-9 (supplier/plant rule, D/S super admin, TB_R_INSTRUCTION, existing ASN tables)
- Prototype: supplier/plant per unit, supplier sees own units, D/S sees all
  with Supplier · Plant column, one-supplier check on Create ASN (MSG9)
- UISS X8/X12/X13/X14/X10 and md: #TEMP_INSTRUCTION pre-mapping,
  TB_R_INSTRUCTION on Create ASN (deleted on Back/Cancel), new
  TB_R_PRA_DAILY_ORDER_MAPPED, ASN into TB_R_DAILY_ORDER_MANIFEST/PART,
  route master and case label/last sequence as existing, cancel from
  source status 2 for held lines
- Executive overview: decided confirmations removed, tasks updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/exec/Crossdock_Executive_Overview.xlsx
+++ b/deliverables/exec/Crossdock_Executive_Overview.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Business Flow" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Executive Summary'!$A$1:$N$31</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Executive Summary'!$A$1:$N$32</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Function Map'!$A$1:$L$22</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Task List'!$A$1:$I$27</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Konfirmasi'!$A$1:$K$32</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Task List'!$A$1:$I$25</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Konfirmasi'!$A$1:$K$23</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'Business Flow'!$A$1:$AN$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -914,7 +914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:M30"/>
+  <dimension ref="B2:M31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -942,7 +942,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>NSP · disusun oleh FID Rayhan (BSA) · status per 15-Oct-2026</t>
+          <t>NSP · disusun oleh FID Rayhan (BSA) · status per 16-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -1030,12 +1030,12 @@
       </c>
       <c r="G11" s="11" t="n"/>
       <c r="H11" s="12">
-        <f>COUNTIF('Task List'!$H$13:$H$26,"&lt;&gt;Done")</f>
+        <f>COUNTIF('Task List'!$H$13:$H$24,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="I11" s="11" t="n"/>
       <c r="J11" s="12">
-        <f>COUNTIF(Konfirmasi!$J$8:$J$31,"Open")</f>
+        <f>COUNTIF(Konfirmasi!$J$8:$J$22,"Open")</f>
         <v/>
       </c>
       <c r="K11" s="11" t="n"/>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
-          <t>▸  Update UISS X8 / X13 setelah konfirmasi case label, isi 1 ASN, route master, tabel ASN (FID Rayhan)</t>
+          <t>▸  Review struktur tabel baru TB_R_INSTRUCTION dan TB_R_PRA_DAILY_ORDER_MAPPED (nama / kolom usulan) (Tim NSP / IT (DBA))</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="H22" s="19" t="inlineStr">
         <is>
-          <t>▸  Finalisasi struktur Pra Daily Order (mapped qty) di UISS X8 / X12 (FID Rayhan)</t>
+          <t>▸  Mapping kolom fisik ke TB_R_DAILY_ORDER_MANIFEST / PART, route master dan last sequence existing (Tim NSP / IT)</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>▸  Tambah kolom HOLD_FLAG / PO_MAPPED_FLAG di H0253 NSP dan cara mempertahankannya saat sync (Tim NSP / IT)</t>
+          <t>▸  Tambah kolom HOLD_FLAG / PO_MAPPED_FLAG di H0253 NSP, dipertahankan saat sync X10 (sudah diputuskan) (Tim NSP / IT)</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="H26" s="19" t="inlineStr">
         <is>
-          <t>▸  Konfirmasi struktur tabel Pra Daily Order dan route master (Tim NSP / IT)</t>
+          <t>▸  Susun testing strategy &amp; test scenario (unit, integration, UAT) X1-X15 (FID Rayhan)</t>
         </is>
       </c>
     </row>
@@ -1234,11 +1234,6 @@
           <t>✔  ASN flow versi 15-Oct: Search (X12 on-demand pre-mapping), Hold Flag per destinasi oleh D/S, Create ASN (mapping), status Ready / Not Ready / Created</t>
         </is>
       </c>
-      <c r="H27" s="19" t="inlineStr">
-        <is>
-          <t>▸  Susun testing strategy &amp; test scenario (unit, integration, UAT) X1-X15 (FID Rayhan)</t>
-        </is>
-      </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="B28" s="19" t="inlineStr">
@@ -1247,8 +1242,15 @@
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="20" t="inlineStr">
+    <row r="29" ht="30" customHeight="1">
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t>✔  Konfirmasi ASN 16-Oct diterapkan: case label &amp; case number sesuai existing, 1 ASN = 1 Supplier + Plant, D/S super admin (semua supplier), route master existing, ASN ke TB_R_DAILY_ORDER_MANIFEST / PART, Create ASN → TB_R_INSTRUCTION (Back / Cancel hapus), tabel baru mapped qty, cancel dari source (status 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="20" t="inlineStr">
         <is>
           <t>Detail: sheet Business Flow (alur), Function Map (X1-X15), Task List, Konfirmasi (keputusan yang dibutuhkan). Prototype: https://ivanrayhannn.github.io/crossdockpoc/</t>
         </is>
@@ -1265,15 +1267,14 @@
     <mergeCell ref="J10:K10"/>
     <mergeCell ref="D15:G15"/>
     <mergeCell ref="H17:M17"/>
+    <mergeCell ref="B29:G29"/>
     <mergeCell ref="H16:M16"/>
     <mergeCell ref="B7:M8"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="H22:M22"/>
-    <mergeCell ref="H27:M27"/>
     <mergeCell ref="F11:G12"/>
     <mergeCell ref="L11:M12"/>
     <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B30:M30"/>
     <mergeCell ref="B24:G24"/>
     <mergeCell ref="H15:M15"/>
     <mergeCell ref="H24:M24"/>
@@ -1287,6 +1288,7 @@
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B22:G22"/>
     <mergeCell ref="B11:C12"/>
+    <mergeCell ref="B31:M31"/>
     <mergeCell ref="D11:E12"/>
     <mergeCell ref="D16:G16"/>
     <mergeCell ref="B27:G27"/>
@@ -1334,7 +1336,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>15 fungsi Crossdock Optimization (UISS X1-X15) · status per 15-Oct-2026</t>
+          <t>15 fungsi Crossdock Optimization (UISS X1-X15) · status per 16-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -1825,7 +1827,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Supplier (detail: D/S team)</t>
+          <t>Supplier / D/S team (super admin)</t>
         </is>
       </c>
       <c r="F14" s="24" t="inlineStr">
@@ -1840,12 +1842,12 @@
       </c>
       <c r="H14" s="24" t="inlineStr">
         <is>
-          <t>Delivery Date, Rit; #TB_R_INSTRUCTION (X12)</t>
+          <t>Delivery Date, Rit (route master); #TEMP_INSTRUCTION (X12)</t>
         </is>
       </c>
       <c r="I14" s="24" t="inlineStr">
         <is>
-          <t>H0253 flags, #TEMP_ASN_DRAFT, Submit ID to X14</t>
+          <t>H0253 flags, TB_R_INSTRUCTION, TB_R_PRA_DAILY_ORDER_MAPPED, Submit ID to X14</t>
         </is>
       </c>
       <c r="J14" s="25" t="inlineStr">
@@ -2068,12 +2070,12 @@
       </c>
       <c r="H18" s="24" t="inlineStr">
         <is>
-          <t>H0253 (status 7, Hold N), Pra Daily Order</t>
+          <t>H0253 (status 7, Hold N), Pra Daily Order, TB_R_PRA_DAILY_ORDER_MAPPED</t>
         </is>
       </c>
       <c r="I18" s="24" t="inlineStr">
         <is>
-          <t>#TB_R_INSTRUCTION (temp, FIFO)</t>
+          <t>#TEMP_INSTRUCTION (temp, FIFO)</t>
         </is>
       </c>
       <c r="J18" s="25" t="inlineStr">
@@ -2125,7 +2127,7 @@
       </c>
       <c r="H19" s="18" t="inlineStr">
         <is>
-          <t>TB_R_ASN_CROSSDOCK_H / _D</t>
+          <t>TB_R_DAILY_ORDER_MANIFEST / _PART (existing)</t>
         </is>
       </c>
       <c r="I19" s="18" t="inlineStr">
@@ -2182,12 +2184,12 @@
       </c>
       <c r="H20" s="24" t="inlineStr">
         <is>
-          <t>#TEMP_ASN_DRAFT, Submit ID</t>
+          <t>TB_R_INSTRUCTION, Submit ID</t>
         </is>
       </c>
       <c r="I20" s="24" t="inlineStr">
         <is>
-          <t>TB_R_ASN_CROSSDOCK_H / _D, log (existing)</t>
+          <t>TB_R_DAILY_ORDER_MANIFEST / _PART (existing), log (existing)</t>
         </is>
       </c>
       <c r="J20" s="25" t="inlineStr">
@@ -2276,7 +2278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I26"/>
+  <dimension ref="B2:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2300,7 +2302,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Pekerjaan yang masih terbuka per 15-Oct-2026. Kolom Status bisa diubah (pilihan list).</t>
+          <t>Pekerjaan yang masih terbuka per 16-Oct-2026. Kolom Status bisa diubah (pilihan list).</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2330,7 @@
         </is>
       </c>
       <c r="D7" s="28">
-        <f>COUNTIF($H$13:$H$26,C7)</f>
+        <f>COUNTIF($H$13:$H$24,C7)</f>
         <v/>
       </c>
     </row>
@@ -2339,7 +2341,7 @@
         </is>
       </c>
       <c r="D8" s="28">
-        <f>COUNTIF($H$13:$H$26,C8)</f>
+        <f>COUNTIF($H$13:$H$24,C8)</f>
         <v/>
       </c>
     </row>
@@ -2350,7 +2352,7 @@
         </is>
       </c>
       <c r="D9" s="28">
-        <f>COUNTIF($H$13:$H$26,C9)</f>
+        <f>COUNTIF($H$13:$H$24,C9)</f>
         <v/>
       </c>
     </row>
@@ -2361,7 +2363,7 @@
         </is>
       </c>
       <c r="D10" s="28">
-        <f>COUNTIF($H$13:$H$26,C10)</f>
+        <f>COUNTIF($H$13:$H$24,C10)</f>
         <v/>
       </c>
     </row>
@@ -2414,32 +2416,32 @@
       </c>
       <c r="C13" s="18" t="inlineStr">
         <is>
-          <t>Update UISS X8 / X13 setelah konfirmasi case label, isi 1 ASN, route master, tabel ASN</t>
+          <t>Review struktur tabel baru TB_R_INSTRUCTION dan TB_R_PRA_DAILY_ORDER_MAPPED (nama / kolom usulan)</t>
         </is>
       </c>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>X8 / X13</t>
+          <t>X8, X12, X14</t>
         </is>
       </c>
       <c r="E13" s="18" t="inlineStr">
         <is>
-          <t>Dokumen</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>FID Rayhan</t>
+          <t>Tim NSP / IT (DBA)</t>
         </is>
       </c>
       <c r="G13" s="18" t="inlineStr">
         <is>
-          <t>Konfirmasi no. 1-5</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H13" s="29" t="inlineStr">
         <is>
-          <t>Waiting confirmation</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="I13" s="22" t="inlineStr">
@@ -2454,32 +2456,32 @@
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t>Finalisasi struktur Pra Daily Order (mapped qty) di UISS X8 / X12</t>
+          <t>Mapping kolom fisik ke TB_R_DAILY_ORDER_MANIFEST / PART, route master dan last sequence existing</t>
         </is>
       </c>
       <c r="D14" s="18" t="inlineStr">
         <is>
-          <t>X8 / X12</t>
+          <t>X8, X13, X14</t>
         </is>
       </c>
       <c r="E14" s="18" t="inlineStr">
         <is>
-          <t>Dokumen</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>FID Rayhan</t>
+          <t>Tim NSP / IT</t>
         </is>
       </c>
       <c r="G14" s="18" t="inlineStr">
         <is>
-          <t>Konfirmasi no. 9</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H14" s="29" t="inlineStr">
         <is>
-          <t>Waiting confirmation</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="I14" s="22" t="inlineStr">
@@ -2514,7 +2516,7 @@
       </c>
       <c r="G15" s="18" t="inlineStr">
         <is>
-          <t>Konfirmasi no. 10-12</t>
+          <t>Konfirmasi no. 1-3</t>
         </is>
       </c>
       <c r="H15" s="29" t="inlineStr">
@@ -2534,7 +2536,7 @@
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>Buat UISS-Batch RPA Sync (jika disetujui)</t>
+          <t>Buat UISS-Batch RPA Sync X16 (jika disetujui)</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
@@ -2554,7 +2556,7 @@
       </c>
       <c r="G16" s="18" t="inlineStr">
         <is>
-          <t>Konfirmasi no. 16-17</t>
+          <t>Konfirmasi no. 7-8</t>
         </is>
       </c>
       <c r="H16" s="29" t="inlineStr">
@@ -2594,7 +2596,7 @@
       </c>
       <c r="G17" s="18" t="inlineStr">
         <is>
-          <t>Konfirmasi no. 20</t>
+          <t>Konfirmasi no. 11</t>
         </is>
       </c>
       <c r="H17" s="29" t="inlineStr">
@@ -2674,7 +2676,7 @@
       </c>
       <c r="G19" s="18" t="inlineStr">
         <is>
-          <t>Konfirmasi no. 15</t>
+          <t>Konfirmasi no. 6</t>
         </is>
       </c>
       <c r="H19" s="29" t="inlineStr">
@@ -2694,7 +2696,7 @@
       </c>
       <c r="C20" s="18" t="inlineStr">
         <is>
-          <t>Tambah kolom HOLD_FLAG / PO_MAPPED_FLAG di H0253 NSP dan cara mempertahankannya saat sync</t>
+          <t>Tambah kolom HOLD_FLAG / PO_MAPPED_FLAG di H0253 NSP, dipertahankan saat sync X10 (sudah diputuskan)</t>
         </is>
       </c>
       <c r="D20" s="18" t="inlineStr">
@@ -2714,7 +2716,7 @@
       </c>
       <c r="G20" s="18" t="inlineStr">
         <is>
-          <t>Konfirmasi no. 7</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H20" s="29" t="inlineStr">
@@ -2734,27 +2736,27 @@
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>Konfirmasi struktur tabel Pra Daily Order dan route master</t>
+          <t>Prototype: Download Case Label sesuai format existing</t>
         </is>
       </c>
       <c r="D21" s="18" t="inlineStr">
         <is>
-          <t>X8, X12</t>
+          <t>X8 / X13</t>
         </is>
       </c>
       <c r="E21" s="18" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Prototype</t>
         </is>
       </c>
       <c r="F21" s="18" t="inlineStr">
         <is>
-          <t>Tim NSP / IT</t>
+          <t>FID Rayhan</t>
         </is>
       </c>
       <c r="G21" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Contoh label existing</t>
         </is>
       </c>
       <c r="H21" s="29" t="inlineStr">
@@ -2764,7 +2766,7 @@
       </c>
       <c r="I21" s="22" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2774,17 +2776,17 @@
       </c>
       <c r="C22" s="18" t="inlineStr">
         <is>
-          <t>Prototype: Download Case Label sesuai format</t>
+          <t>Susun testing strategy &amp; test scenario (unit, integration, UAT) X1-X15</t>
         </is>
       </c>
       <c r="D22" s="18" t="inlineStr">
         <is>
-          <t>X8 / X13</t>
+          <t>X1-X15</t>
         </is>
       </c>
       <c r="E22" s="18" t="inlineStr">
         <is>
-          <t>Prototype</t>
+          <t>Testing</t>
         </is>
       </c>
       <c r="F22" s="18" t="inlineStr">
@@ -2794,17 +2796,17 @@
       </c>
       <c r="G22" s="18" t="inlineStr">
         <is>
-          <t>Konfirmasi no. 1</t>
+          <t>UISS final</t>
         </is>
       </c>
       <c r="H22" s="29" t="inlineStr">
         <is>
-          <t>Waiting confirmation</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="I22" s="22" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2814,37 +2816,37 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>Prototype: Cancel ASN di ASN Inquiry (jika diperlukan)</t>
+          <t>Definisikan proses lanjutan setelah ASN (penerimaan di crossdock, pengiriman ke destinasi)</t>
         </is>
       </c>
       <c r="D23" s="18" t="inlineStr">
         <is>
-          <t>X13</t>
+          <t>Next scope</t>
         </is>
       </c>
       <c r="E23" s="18" t="inlineStr">
         <is>
-          <t>Prototype</t>
+          <t>Analisis</t>
         </is>
       </c>
       <c r="F23" s="18" t="inlineStr">
         <is>
-          <t>FID Rayhan</t>
+          <t>FID Rayhan / User</t>
         </is>
       </c>
       <c r="G23" s="18" t="inlineStr">
         <is>
-          <t>Konfirmasi no. 8</t>
+          <t>Arahan user</t>
         </is>
       </c>
       <c r="H23" s="29" t="inlineStr">
         <is>
-          <t>Waiting confirmation</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="I23" s="22" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2854,17 +2856,17 @@
       </c>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>Susun testing strategy &amp; test scenario (unit, integration, UAT) X1-X15</t>
+          <t>Susun BRD / TSD (jika dibutuhkan proyek)</t>
         </is>
       </c>
       <c r="D24" s="18" t="inlineStr">
         <is>
-          <t>X1-X15</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E24" s="18" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Dokumen</t>
         </is>
       </c>
       <c r="F24" s="18" t="inlineStr">
@@ -2874,7 +2876,7 @@
       </c>
       <c r="G24" s="18" t="inlineStr">
         <is>
-          <t>UISS final</t>
+          <t>Arahan user</t>
         </is>
       </c>
       <c r="H24" s="29" t="inlineStr">
@@ -2884,98 +2886,18 @@
       </c>
       <c r="I24" s="22" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="B25" s="22" t="n">
-        <v>13</v>
-      </c>
-      <c r="C25" s="18" t="inlineStr">
-        <is>
-          <t>Definisikan proses lanjutan setelah ASN (penerimaan di crossdock, pengiriman ke destinasi)</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>Next scope</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>Analisis</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>FID Rayhan / User</t>
-        </is>
-      </c>
-      <c r="G25" s="18" t="inlineStr">
-        <is>
-          <t>Arahan user</t>
-        </is>
-      </c>
-      <c r="H25" s="29" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I25" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="B26" s="22" t="n">
-        <v>14</v>
-      </c>
-      <c r="C26" s="18" t="inlineStr">
-        <is>
-          <t>Susun BRD / TSD (jika dibutuhkan proyek)</t>
-        </is>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>Dokumen</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>FID Rayhan</t>
-        </is>
-      </c>
-      <c r="G26" s="18" t="inlineStr">
-        <is>
-          <t>Arahan user</t>
-        </is>
-      </c>
-      <c r="H26" s="29" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I26" s="22" t="inlineStr">
-        <is>
           <t>Low</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I13:I26">
+  <conditionalFormatting sqref="I13:I24">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"High"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not started,Waiting confirmation,In progress,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2991,7 +2913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K31"/>
+  <dimension ref="B2:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -3016,7 +2938,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Pertanyaan yang perlu keputusan user per 15-Oct-2026.</t>
+          <t>Pertanyaan yang perlu keputusan user per 16-Oct-2026.</t>
         </is>
       </c>
     </row>
@@ -3092,27 +3014,27 @@
       </c>
       <c r="C8" s="22" t="inlineStr">
         <is>
-          <t>X8 / X13</t>
+          <t>X9-X11</t>
         </is>
       </c>
       <c r="D8" s="17" t="inlineStr">
         <is>
-          <t>Case label</t>
+          <t>Jadwal &amp; retry</t>
         </is>
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>Format, isi, dan nama file case label (Download Case Label).</t>
+          <t>Jadwal scheduler NSP untuk X9, X10, X11 dan perlu auto retry seperti X6 / X7?</t>
         </is>
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Ikuti format case label NSP existing.</t>
+          <t>Setelah data G-TOPAS tersedia; auto retry 3x.</t>
         </is>
       </c>
       <c r="G8" s="18" t="inlineStr">
         <is>
-          <t>Case label belum bisa dicetak; UISS X8 / X13 masih TBD.</t>
+          <t>Schedule sheet di UISS masih TBC.</t>
         </is>
       </c>
       <c r="H8" s="30" t="n"/>
@@ -3128,27 +3050,27 @@
       </c>
       <c r="C9" s="22" t="inlineStr">
         <is>
-          <t>X8</t>
+          <t>X5</t>
         </is>
       </c>
       <c r="D9" s="17" t="inlineStr">
         <is>
-          <t>Isi 1 ASN</t>
+          <t>Jadwal X5</t>
         </is>
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>Apakah 1 ASN wajib 1 supplier / plant?</t>
+          <t>Tanggal / jam scheduler bulanan X5.</t>
         </is>
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>Ya, 1 ASN = 1 supplier + plant.</t>
+          <t>Tanggal 1 jam 01:00, sebelum X6.</t>
         </is>
       </c>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>Validasi pilihan unit di Create ASN.</t>
+          <t>Schedule sheet X5 / X6.</t>
         </is>
       </c>
       <c r="H9" s="30" t="n"/>
@@ -3164,27 +3086,27 @@
       </c>
       <c r="C10" s="22" t="inlineStr">
         <is>
-          <t>X8</t>
+          <t>X5 / X6</t>
         </is>
       </c>
       <c r="D10" s="17" t="inlineStr">
         <is>
-          <t>Akses D/S</t>
+          <t>X5 gagal</t>
         </is>
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>Apakah tim D/S juga boleh Create / Submit ASN, atau hanya melihat + hold?</t>
+          <t>Kalau X5 gagal, apakah X6 dibatalkan?</t>
         </is>
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>Hanya melihat + hold.</t>
+          <t>Ya, X6 tidak jalan.</t>
         </is>
       </c>
       <c r="G10" s="18" t="inlineStr">
         <is>
-          <t>Hak akses tombol Create ASN.</t>
+          <t>Aturan dependensi batch.</t>
         </is>
       </c>
       <c r="H10" s="30" t="n"/>
@@ -3200,27 +3122,27 @@
       </c>
       <c r="C11" s="22" t="inlineStr">
         <is>
-          <t>X8</t>
+          <t>X5</t>
         </is>
       </c>
       <c r="D11" s="17" t="inlineStr">
         <is>
-          <t>Route master</t>
+          <t>Kolom DAD</t>
         </is>
       </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>Nama dan struktur tabel route master (Rit / Route).</t>
+          <t>Kolom DAD di Actual Demand Summary dipakai atau tidak?</t>
         </is>
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>Pakai route master NSP existing.</t>
+          <t>Tidak dipakai (hanya MAD).</t>
         </is>
       </c>
       <c r="G11" s="18" t="inlineStr">
         <is>
-          <t>Combo Rit masih mock.</t>
+          <t>Mapping kolom X5.</t>
         </is>
       </c>
       <c r="H11" s="30" t="n"/>
@@ -3236,27 +3158,27 @@
       </c>
       <c r="C12" s="22" t="inlineStr">
         <is>
-          <t>X8 / X13</t>
+          <t>X5 / X7</t>
         </is>
       </c>
       <c r="D12" s="17" t="inlineStr">
         <is>
-          <t>Tabel ASN</t>
+          <t>Order type N + S</t>
         </is>
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>Konfirmasi TB_R_ASN_CROSSDOCK_H / _D (usulan) atau pakai tabel ASN existing.</t>
+          <t>ORDER_TYPE_GROUP N dan S dijumlahkan (sementara). Final?</t>
         </is>
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>Pakai usulan di Appendix UISS X8.</t>
+          <t>Tetap dijumlahkan.</t>
         </is>
       </c>
       <c r="G12" s="18" t="inlineStr">
         <is>
-          <t>Data mapping Submit ASN.</t>
+          <t>Rumus MAD di X6 / X7.</t>
         </is>
       </c>
       <c r="H12" s="30" t="n"/>
@@ -3272,27 +3194,27 @@
       </c>
       <c r="C13" s="22" t="inlineStr">
         <is>
-          <t>X8</t>
+          <t>X10</t>
         </is>
       </c>
       <c r="D13" s="17" t="inlineStr">
         <is>
-          <t>Back / Cancel</t>
+          <t>SERIAL_NO</t>
         </is>
       </c>
       <c r="E13" s="18" t="inlineStr">
         <is>
-          <t>Back / Cancel di Case List melepas mapping (PO_MAPPED_FLAG dan qty PO kembali). Setuju?</t>
+          <t>SERIAL_NO perlu ditambahkan di tabel / query H0253 sumber (DB Surrounding).</t>
         </is>
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>Ya.</t>
+          <t>Tim surrounding menambah kolom.</t>
         </is>
       </c>
       <c r="G13" s="18" t="inlineStr">
         <is>
-          <t>Order bisa terkunci tanpa ASN.</t>
+          <t>Tanpa SERIAL_NO key H0253 tidak unik.</t>
         </is>
       </c>
       <c r="H13" s="30" t="n"/>
@@ -3308,27 +3230,27 @@
       </c>
       <c r="C14" s="22" t="inlineStr">
         <is>
-          <t>X10</t>
+          <t>X3</t>
         </is>
       </c>
       <c r="D14" s="17" t="inlineStr">
         <is>
-          <t>Flag H0253</t>
+          <t>RPA Sync</t>
         </is>
       </c>
       <c r="E14" s="18" t="inlineStr">
         <is>
-          <t>HOLD_FLAG dan PO_MAPPED_FLAG dipertahankan per unique key saat delete - insert X10. Setuju?</t>
+          <t>Detail fungsi RPA: layar global system, urutan input, waktu proses, timeout, user ID RPA.</t>
         </is>
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>Ya (cara teknis oleh tim IT).</t>
+          <t>Perlu sesi dengan tim RPA.</t>
         </is>
       </c>
       <c r="G14" s="18" t="inlineStr">
         <is>
-          <t>Hold / mapping hilang setiap sync.</t>
+          <t>UISS RPA belum bisa dibuat.</t>
         </is>
       </c>
       <c r="H14" s="30" t="n"/>
@@ -3344,27 +3266,27 @@
       </c>
       <c r="C15" s="22" t="inlineStr">
         <is>
-          <t>X13</t>
+          <t>X3</t>
         </is>
       </c>
       <c r="D15" s="17" t="inlineStr">
         <is>
-          <t>Cancel ASN</t>
+          <t>UISS RPA</t>
         </is>
       </c>
       <c r="E15" s="18" t="inlineStr">
         <is>
-          <t>Perlu cancel / revisi ASN dari ASN Inquiry?</t>
+          <t>Perlu UISS-Batch tersendiri untuk RPA Sync?</t>
         </is>
       </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>Perlu cancel selama barang belum dikirim.</t>
+          <t>Ya, X16.</t>
         </is>
       </c>
       <c r="G15" s="18" t="inlineStr">
         <is>
-          <t>Tambahan fungsi dan status ASN.</t>
+          <t>Tambahan dokumen.</t>
         </is>
       </c>
       <c r="H15" s="30" t="n"/>
@@ -3380,27 +3302,27 @@
       </c>
       <c r="C16" s="22" t="inlineStr">
         <is>
-          <t>X8 / X12</t>
+          <t>X3</t>
         </is>
       </c>
       <c r="D16" s="17" t="inlineStr">
         <is>
-          <t>Pra Daily Order</t>
+          <t>Status Waiting</t>
         </is>
       </c>
       <c r="E16" s="18" t="inlineStr">
         <is>
-          <t>Struktur fisik TB_R_PRA_DAILY_ORDER_MANIFEST / PART dan kolom qty terpakai (mapped qty).</t>
+          <t>Apakah status Waiting (Sync) perlu batas waktu, lalu kembali ke Failed?</t>
         </is>
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>Tambah kolom MAPPED_QTY di PART.</t>
+          <t>Ya, 30 menit.</t>
         </is>
       </c>
       <c r="G16" s="18" t="inlineStr">
         <is>
-          <t>Logika FIFO X12 / Create ASN belum final.</t>
+          <t>Status sync bisa menggantung.</t>
         </is>
       </c>
       <c r="H16" s="30" t="n"/>
@@ -3416,27 +3338,27 @@
       </c>
       <c r="C17" s="22" t="inlineStr">
         <is>
-          <t>X9-X11</t>
+          <t>X1-X4</t>
         </is>
       </c>
       <c r="D17" s="17" t="inlineStr">
         <is>
-          <t>Jadwal &amp; retry</t>
+          <t>History</t>
         </is>
       </c>
       <c r="E17" s="18" t="inlineStr">
         <is>
-          <t>Jadwal scheduler NSP untuk X9, X10, X11 dan perlu auto retry seperti X6 / X7?</t>
+          <t>Konfirmasi kolom dan retensi TB_H_PART_CANDIDATE (usulan 24 bulan).</t>
         </is>
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>Setelah data G-TOPAS tersedia; auto retry 3x.</t>
+          <t>Pakai usulan.</t>
         </is>
       </c>
       <c r="G17" s="18" t="inlineStr">
         <is>
-          <t>Schedule sheet di UISS masih TBC.</t>
+          <t>Appendix tabel history.</t>
         </is>
       </c>
       <c r="H17" s="30" t="n"/>
@@ -3452,27 +3374,27 @@
       </c>
       <c r="C18" s="22" t="inlineStr">
         <is>
-          <t>X5</t>
+          <t>X1-X4</t>
         </is>
       </c>
       <c r="D18" s="17" t="inlineStr">
         <is>
-          <t>Jadwal X5</t>
+          <t>Panjang kolom</t>
         </is>
       </c>
       <c r="E18" s="18" t="inlineStr">
         <is>
-          <t>Tanggal / jam scheduler bulanan X5.</t>
+          <t>Panjang VARCHAR kolom (PART_NO dll.) dan nama field Part Name di TB_M_PART_MASTER.</t>
         </is>
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>Tanggal 1 jam 01:00, sebelum X6.</t>
+          <t>Ikuti TB_M_PART_MASTER.</t>
         </is>
       </c>
       <c r="G18" s="18" t="inlineStr">
         <is>
-          <t>Schedule sheet X5 / X6.</t>
+          <t>Masih VARCHAR(TBD) di Appendix.</t>
         </is>
       </c>
       <c r="H18" s="30" t="n"/>
@@ -3488,27 +3410,27 @@
       </c>
       <c r="C19" s="22" t="inlineStr">
         <is>
-          <t>X5 / X6</t>
+          <t>X2 / X4</t>
         </is>
       </c>
       <c r="D19" s="17" t="inlineStr">
         <is>
-          <t>X5 gagal</t>
+          <t>Template &amp; log</t>
         </is>
       </c>
       <c r="E19" s="18" t="inlineStr">
         <is>
-          <t>Kalau X5 gagal, apakah X6 dibatalkan?</t>
+          <t>Lokasi file template dan result report; retensi Log upload.</t>
         </is>
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>Ya, X6 tidak jalan.</t>
+          <t>Shared folder NSP; retensi 12 bulan.</t>
         </is>
       </c>
       <c r="G19" s="18" t="inlineStr">
         <is>
-          <t>Aturan dependensi batch.</t>
+          <t>Operation description upload.</t>
         </is>
       </c>
       <c r="H19" s="30" t="n"/>
@@ -3524,27 +3446,27 @@
       </c>
       <c r="C20" s="22" t="inlineStr">
         <is>
-          <t>X5</t>
+          <t>X1</t>
         </is>
       </c>
       <c r="D20" s="17" t="inlineStr">
         <is>
-          <t>Kolom DAD</t>
+          <t>Akun read only</t>
         </is>
       </c>
       <c r="E20" s="18" t="inlineStr">
         <is>
-          <t>Kolom DAD di Actual Demand Summary dipakai atau tidak?</t>
+          <t>Definisi akun read-only ([View]) untuk Part List.</t>
         </is>
       </c>
       <c r="F20" s="18" t="inlineStr">
         <is>
-          <t>Tidak dipakai (hanya MAD).</t>
+          <t>Role Viewer: hanya Search / Export.</t>
         </is>
       </c>
       <c r="G20" s="18" t="inlineStr">
         <is>
-          <t>Mapping kolom X5.</t>
+          <t>Screen mode View.</t>
         </is>
       </c>
       <c r="H20" s="30" t="n"/>
@@ -3560,27 +3482,27 @@
       </c>
       <c r="C21" s="22" t="inlineStr">
         <is>
-          <t>X5 / X7</t>
+          <t>X15</t>
         </is>
       </c>
       <c r="D21" s="17" t="inlineStr">
         <is>
-          <t>Order type N + S</t>
+          <t>Menu Settings</t>
         </is>
       </c>
       <c r="E21" s="18" t="inlineStr">
         <is>
-          <t>ORDER_TYPE_GROUP N dan S dijumlahkan (sementara). Final?</t>
+          <t>Pengaturan show / hide menu berlaku per role atau global, dan siapa yang boleh membuka layar ini?</t>
         </is>
       </c>
       <c r="F21" s="18" t="inlineStr">
         <is>
-          <t>Tetap dijumlahkan.</t>
+          <t>Per role; hanya admin.</t>
         </is>
       </c>
       <c r="G21" s="18" t="inlineStr">
         <is>
-          <t>Rumus MAD di X6 / X7.</t>
+          <t>Struktur TB_M_MENU_VISIBILITY.</t>
         </is>
       </c>
       <c r="H21" s="30" t="n"/>
@@ -3596,27 +3518,27 @@
       </c>
       <c r="C22" s="22" t="inlineStr">
         <is>
-          <t>X10</t>
+          <t>X1</t>
         </is>
       </c>
       <c r="D22" s="17" t="inlineStr">
         <is>
-          <t>SERIAL_NO</t>
+          <t>Effective Start Date</t>
         </is>
       </c>
       <c r="E22" s="18" t="inlineStr">
         <is>
-          <t>SERIAL_NO perlu ditambahkan di tabel / query H0253 sumber (DB Surrounding).</t>
+          <t>Kalimat "Effective Start Date" yang menggantung di Op Desc 5.4 a.4 (UISS X1): aturan apa yang dimaksud?</t>
         </is>
       </c>
       <c r="F22" s="18" t="inlineStr">
         <is>
-          <t>Tim surrounding menambah kolom.</t>
+          <t>Default besok, minimum hari ini, wajib diisi.</t>
         </is>
       </c>
       <c r="G22" s="18" t="inlineStr">
         <is>
-          <t>Tanpa SERIAL_NO key H0253 tidak unik.</t>
+          <t>Op Desc X1 belum lengkap.</t>
         </is>
       </c>
       <c r="H22" s="30" t="n"/>
@@ -3626,332 +3548,8 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="42" customHeight="1">
-      <c r="B23" s="22" t="n">
-        <v>16</v>
-      </c>
-      <c r="C23" s="22" t="inlineStr">
-        <is>
-          <t>X3</t>
-        </is>
-      </c>
-      <c r="D23" s="17" t="inlineStr">
-        <is>
-          <t>RPA Sync</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>Detail fungsi RPA: layar global system, urutan input, waktu proses, timeout, user ID RPA.</t>
-        </is>
-      </c>
-      <c r="F23" s="18" t="inlineStr">
-        <is>
-          <t>Perlu sesi dengan tim RPA.</t>
-        </is>
-      </c>
-      <c r="G23" s="18" t="inlineStr">
-        <is>
-          <t>UISS RPA belum bisa dibuat.</t>
-        </is>
-      </c>
-      <c r="H23" s="30" t="n"/>
-      <c r="I23" s="30" t="n"/>
-      <c r="J23" s="31">
-        <f>IF(H23="","Open","Decided")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="42" customHeight="1">
-      <c r="B24" s="22" t="n">
-        <v>17</v>
-      </c>
-      <c r="C24" s="22" t="inlineStr">
-        <is>
-          <t>X3</t>
-        </is>
-      </c>
-      <c r="D24" s="17" t="inlineStr">
-        <is>
-          <t>UISS RPA</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>Perlu UISS-Batch tersendiri untuk RPA Sync?</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>Ya, X14.</t>
-        </is>
-      </c>
-      <c r="G24" s="18" t="inlineStr">
-        <is>
-          <t>Tambahan dokumen.</t>
-        </is>
-      </c>
-      <c r="H24" s="30" t="n"/>
-      <c r="I24" s="30" t="n"/>
-      <c r="J24" s="31">
-        <f>IF(H24="","Open","Decided")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="42" customHeight="1">
-      <c r="B25" s="22" t="n">
-        <v>18</v>
-      </c>
-      <c r="C25" s="22" t="inlineStr">
-        <is>
-          <t>X3</t>
-        </is>
-      </c>
-      <c r="D25" s="17" t="inlineStr">
-        <is>
-          <t>Status Waiting</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>Apakah status Waiting (Sync) perlu batas waktu, lalu kembali ke Failed?</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>Ya, 30 menit.</t>
-        </is>
-      </c>
-      <c r="G25" s="18" t="inlineStr">
-        <is>
-          <t>Status sync bisa menggantung.</t>
-        </is>
-      </c>
-      <c r="H25" s="30" t="n"/>
-      <c r="I25" s="30" t="n"/>
-      <c r="J25" s="31">
-        <f>IF(H25="","Open","Decided")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="42" customHeight="1">
-      <c r="B26" s="22" t="n">
-        <v>19</v>
-      </c>
-      <c r="C26" s="22" t="inlineStr">
-        <is>
-          <t>X1-X4</t>
-        </is>
-      </c>
-      <c r="D26" s="17" t="inlineStr">
-        <is>
-          <t>History</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>Konfirmasi kolom dan retensi TB_H_PART_CANDIDATE (usulan 24 bulan).</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>Pakai usulan.</t>
-        </is>
-      </c>
-      <c r="G26" s="18" t="inlineStr">
-        <is>
-          <t>Appendix tabel history.</t>
-        </is>
-      </c>
-      <c r="H26" s="30" t="n"/>
-      <c r="I26" s="30" t="n"/>
-      <c r="J26" s="31">
-        <f>IF(H26="","Open","Decided")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="42" customHeight="1">
-      <c r="B27" s="22" t="n">
-        <v>20</v>
-      </c>
-      <c r="C27" s="22" t="inlineStr">
-        <is>
-          <t>X1-X4</t>
-        </is>
-      </c>
-      <c r="D27" s="17" t="inlineStr">
-        <is>
-          <t>Panjang kolom</t>
-        </is>
-      </c>
-      <c r="E27" s="18" t="inlineStr">
-        <is>
-          <t>Panjang VARCHAR kolom (PART_NO dll.) dan nama field Part Name di TB_M_PART_MASTER.</t>
-        </is>
-      </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>Ikuti TB_M_PART_MASTER.</t>
-        </is>
-      </c>
-      <c r="G27" s="18" t="inlineStr">
-        <is>
-          <t>Masih VARCHAR(TBD) di Appendix.</t>
-        </is>
-      </c>
-      <c r="H27" s="30" t="n"/>
-      <c r="I27" s="30" t="n"/>
-      <c r="J27" s="31">
-        <f>IF(H27="","Open","Decided")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="42" customHeight="1">
-      <c r="B28" s="22" t="n">
-        <v>21</v>
-      </c>
-      <c r="C28" s="22" t="inlineStr">
-        <is>
-          <t>X2 / X4</t>
-        </is>
-      </c>
-      <c r="D28" s="17" t="inlineStr">
-        <is>
-          <t>Template &amp; log</t>
-        </is>
-      </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>Lokasi file template dan result report; retensi Log upload.</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>Shared folder NSP; retensi 12 bulan.</t>
-        </is>
-      </c>
-      <c r="G28" s="18" t="inlineStr">
-        <is>
-          <t>Operation description upload.</t>
-        </is>
-      </c>
-      <c r="H28" s="30" t="n"/>
-      <c r="I28" s="30" t="n"/>
-      <c r="J28" s="31">
-        <f>IF(H28="","Open","Decided")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="42" customHeight="1">
-      <c r="B29" s="22" t="n">
-        <v>22</v>
-      </c>
-      <c r="C29" s="22" t="inlineStr">
-        <is>
-          <t>X1</t>
-        </is>
-      </c>
-      <c r="D29" s="17" t="inlineStr">
-        <is>
-          <t>Akun read only</t>
-        </is>
-      </c>
-      <c r="E29" s="18" t="inlineStr">
-        <is>
-          <t>Definisi akun read-only ([View]) untuk Part List.</t>
-        </is>
-      </c>
-      <c r="F29" s="18" t="inlineStr">
-        <is>
-          <t>Role Viewer: hanya Search / Export.</t>
-        </is>
-      </c>
-      <c r="G29" s="18" t="inlineStr">
-        <is>
-          <t>Screen mode View.</t>
-        </is>
-      </c>
-      <c r="H29" s="30" t="n"/>
-      <c r="I29" s="30" t="n"/>
-      <c r="J29" s="31">
-        <f>IF(H29="","Open","Decided")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="42" customHeight="1">
-      <c r="B30" s="22" t="n">
-        <v>23</v>
-      </c>
-      <c r="C30" s="22" t="inlineStr">
-        <is>
-          <t>X15</t>
-        </is>
-      </c>
-      <c r="D30" s="17" t="inlineStr">
-        <is>
-          <t>Menu Settings</t>
-        </is>
-      </c>
-      <c r="E30" s="18" t="inlineStr">
-        <is>
-          <t>Pengaturan show / hide menu berlaku per role atau global, dan siapa yang boleh membuka layar ini?</t>
-        </is>
-      </c>
-      <c r="F30" s="18" t="inlineStr">
-        <is>
-          <t>Per role; hanya admin.</t>
-        </is>
-      </c>
-      <c r="G30" s="18" t="inlineStr">
-        <is>
-          <t>Struktur TB_M_MENU_VISIBILITY.</t>
-        </is>
-      </c>
-      <c r="H30" s="30" t="n"/>
-      <c r="I30" s="30" t="n"/>
-      <c r="J30" s="31">
-        <f>IF(H30="","Open","Decided")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="42" customHeight="1">
-      <c r="B31" s="22" t="n">
-        <v>24</v>
-      </c>
-      <c r="C31" s="22" t="inlineStr">
-        <is>
-          <t>X1</t>
-        </is>
-      </c>
-      <c r="D31" s="17" t="inlineStr">
-        <is>
-          <t>Effective Start Date</t>
-        </is>
-      </c>
-      <c r="E31" s="18" t="inlineStr">
-        <is>
-          <t>Kalimat "Effective Start Date" yang menggantung di Op Desc 5.4 a.4 (UISS X1): aturan apa yang dimaksud?</t>
-        </is>
-      </c>
-      <c r="F31" s="18" t="inlineStr">
-        <is>
-          <t>Default besok, minimum hari ini, wajib diisi.</t>
-        </is>
-      </c>
-      <c r="G31" s="18" t="inlineStr">
-        <is>
-          <t>Op Desc X1 belum lengkap.</t>
-        </is>
-      </c>
-      <c r="H31" s="30" t="n"/>
-      <c r="I31" s="30" t="n"/>
-      <c r="J31" s="31">
-        <f>IF(H31="","Open","Decided")</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="J8:J31">
+  <conditionalFormatting sqref="J8:J22">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Open"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Rename systems: G-TOPAS to T-System, NSP to Supplier System
Prototype (header, sidebar, footer, pages), UISS builders and all UISS
X1-X15, md files and executive overview. Column names and internal keys
are unchanged. Screenshots retaken.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/exec/Crossdock_Executive_Overview.xlsx
+++ b/deliverables/exec/Crossdock_Executive_Overview.xlsx
@@ -942,7 +942,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>NSP · disusun oleh FID Rayhan (BSA) · status per 16-Oct-2026</t>
+          <t>Supplier System · disusun oleh FID Rayhan (BSA) · status per 16-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
-          <t>▸  Review struktur tabel baru TB_R_INSTRUCTION dan TB_R_PRA_DAILY_ORDER_MAPPED (nama / kolom usulan) (Tim NSP / IT (DBA))</t>
+          <t>▸  Review struktur tabel baru TB_R_INSTRUCTION dan TB_R_PRA_DAILY_ORDER_MAPPED (nama / kolom usulan) (Tim Supplier System / IT (DBA))</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="H22" s="19" t="inlineStr">
         <is>
-          <t>▸  Mapping kolom fisik ke TB_R_DAILY_ORDER_MANIFEST / PART, route master dan last sequence existing (Tim NSP / IT)</t>
+          <t>▸  Mapping kolom fisik ke TB_R_DAILY_ORDER_MANIFEST / PART, route master dan last sequence existing (Tim Supplier System / IT)</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1195,7 @@
     <row r="24" ht="30" customHeight="1">
       <c r="B24" s="19" t="inlineStr">
         <is>
-          <t>✔  Struktur tabel H0202 / H0253 / H0125 dari I/F layout G-TOPAS, termasuk SERIAL_NO</t>
+          <t>✔  Struktur tabel H0202 / H0253 / H0125 dari I/F layout T-System, termasuk SERIAL_NO</t>
         </is>
       </c>
       <c r="H24" s="19" t="inlineStr">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>▸  Tambah kolom HOLD_FLAG / PO_MAPPED_FLAG di H0253 NSP, dipertahankan saat sync X10 (sudah diputuskan) (Tim NSP / IT)</t>
+          <t>▸  Tambah kolom HOLD_FLAG / PO_MAPPED_FLAG di H0253 Supplier System, dipertahankan saat sync X10 (sudah diputuskan) (Tim Supplier System / IT)</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="I11" s="18" t="inlineStr">
         <is>
-          <t>NSP TB_R_ACTUAL_DEMAND_SUMMARY</t>
+          <t>Supplier System TB_R_ACTUAL_DEMAND_SUMMARY</t>
         </is>
       </c>
       <c r="J11" s="22" t="inlineStr">
@@ -1899,12 +1899,12 @@
       </c>
       <c r="H15" s="18" t="inlineStr">
         <is>
-          <t>G-TOPAS H0202</t>
+          <t>T-System H0202</t>
         </is>
       </c>
       <c r="I15" s="18" t="inlineStr">
         <is>
-          <t>NSP TB_R_H0202</t>
+          <t>Supplier System TB_R_H0202</t>
         </is>
       </c>
       <c r="J15" s="22" t="inlineStr">
@@ -1956,12 +1956,12 @@
       </c>
       <c r="H16" s="24" t="inlineStr">
         <is>
-          <t>G-TOPAS H0253</t>
+          <t>T-System H0253</t>
         </is>
       </c>
       <c r="I16" s="24" t="inlineStr">
         <is>
-          <t>NSP TB_R_H0253_ORDER_CONTROL_PRE</t>
+          <t>Supplier System TB_R_H0253_ORDER_CONTROL_PRE</t>
         </is>
       </c>
       <c r="J16" s="25" t="inlineStr">
@@ -2013,12 +2013,12 @@
       </c>
       <c r="H17" s="18" t="inlineStr">
         <is>
-          <t>G-TOPAS H0125</t>
+          <t>T-System H0125</t>
         </is>
       </c>
       <c r="I17" s="18" t="inlineStr">
         <is>
-          <t>NSP TB_M_H0125_DESTINATION</t>
+          <t>Supplier System TB_M_H0125_DESTINATION</t>
         </is>
       </c>
       <c r="J17" s="22" t="inlineStr">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>Tim NSP / IT (DBA)</t>
+          <t>Tim Supplier System / IT (DBA)</t>
         </is>
       </c>
       <c r="G13" s="18" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>Tim NSP / IT</t>
+          <t>Tim Supplier System / IT</t>
         </is>
       </c>
       <c r="G14" s="18" t="inlineStr">
@@ -2696,7 +2696,7 @@
       </c>
       <c r="C20" s="18" t="inlineStr">
         <is>
-          <t>Tambah kolom HOLD_FLAG / PO_MAPPED_FLAG di H0253 NSP, dipertahankan saat sync X10 (sudah diputuskan)</t>
+          <t>Tambah kolom HOLD_FLAG / PO_MAPPED_FLAG di H0253 Supplier System, dipertahankan saat sync X10 (sudah diputuskan)</t>
         </is>
       </c>
       <c r="D20" s="18" t="inlineStr">
@@ -2711,7 +2711,7 @@
       </c>
       <c r="F20" s="18" t="inlineStr">
         <is>
-          <t>Tim NSP / IT</t>
+          <t>Tim Supplier System / IT</t>
         </is>
       </c>
       <c r="G20" s="18" t="inlineStr">
@@ -3024,12 +3024,12 @@
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>Jadwal scheduler NSP untuk X9, X10, X11 dan perlu auto retry seperti X6 / X7?</t>
+          <t>Jadwal scheduler Supplier System untuk X9, X10, X11 dan perlu auto retry seperti X6 / X7?</t>
         </is>
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Setelah data G-TOPAS tersedia; auto retry 3x.</t>
+          <t>Setelah data T-System tersedia; auto retry 3x.</t>
         </is>
       </c>
       <c r="G8" s="18" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>Shared folder NSP; retensi 12 bulan.</t>
+          <t>Shared folder Supplier System; retensi 12 bulan.</t>
         </is>
       </c>
       <c r="G19" s="18" t="inlineStr">
@@ -3687,7 +3687,7 @@
     <row r="8" ht="9" customHeight="1">
       <c r="B8" s="34" t="inlineStr">
         <is>
-          <t>G-TOPAS /
+          <t>T-System /
 DB Surrounding</t>
         </is>
       </c>
@@ -3936,7 +3936,7 @@
     <row r="13" ht="9" customHeight="1">
       <c r="B13" s="45" t="inlineStr">
         <is>
-          <t>NSP Batch
+          <t>Supplier System Batch
 (System)</t>
         </is>
       </c>
@@ -4002,7 +4002,7 @@
               <sz val="9"/>
             </rPr>
             <t>Replicate data
-to NSP</t>
+to Supplier System</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
Keep G-TOPAS and NSP names in UISS and documents
The system rename (T-System, Supplier System) applies to the web
prototype only. UISS X1-X15, builders, screenshots, md and executive
overview are restored to the previous names.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/exec/Crossdock_Executive_Overview.xlsx
+++ b/deliverables/exec/Crossdock_Executive_Overview.xlsx
@@ -942,7 +942,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Supplier System · disusun oleh FID Rayhan (BSA) · status per 16-Oct-2026</t>
+          <t>NSP · disusun oleh FID Rayhan (BSA) · status per 16-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
-          <t>▸  Review struktur tabel baru TB_R_INSTRUCTION dan TB_R_PRA_DAILY_ORDER_MAPPED (nama / kolom usulan) (Tim Supplier System / IT (DBA))</t>
+          <t>▸  Review struktur tabel baru TB_R_INSTRUCTION dan TB_R_PRA_DAILY_ORDER_MAPPED (nama / kolom usulan) (Tim NSP / IT (DBA))</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="H22" s="19" t="inlineStr">
         <is>
-          <t>▸  Mapping kolom fisik ke TB_R_DAILY_ORDER_MANIFEST / PART, route master dan last sequence existing (Tim Supplier System / IT)</t>
+          <t>▸  Mapping kolom fisik ke TB_R_DAILY_ORDER_MANIFEST / PART, route master dan last sequence existing (Tim NSP / IT)</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1195,7 @@
     <row r="24" ht="30" customHeight="1">
       <c r="B24" s="19" t="inlineStr">
         <is>
-          <t>✔  Struktur tabel H0202 / H0253 / H0125 dari I/F layout T-System, termasuk SERIAL_NO</t>
+          <t>✔  Struktur tabel H0202 / H0253 / H0125 dari I/F layout G-TOPAS, termasuk SERIAL_NO</t>
         </is>
       </c>
       <c r="H24" s="19" t="inlineStr">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>▸  Tambah kolom HOLD_FLAG / PO_MAPPED_FLAG di H0253 Supplier System, dipertahankan saat sync X10 (sudah diputuskan) (Tim Supplier System / IT)</t>
+          <t>▸  Tambah kolom HOLD_FLAG / PO_MAPPED_FLAG di H0253 NSP, dipertahankan saat sync X10 (sudah diputuskan) (Tim NSP / IT)</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="I11" s="18" t="inlineStr">
         <is>
-          <t>Supplier System TB_R_ACTUAL_DEMAND_SUMMARY</t>
+          <t>NSP TB_R_ACTUAL_DEMAND_SUMMARY</t>
         </is>
       </c>
       <c r="J11" s="22" t="inlineStr">
@@ -1899,12 +1899,12 @@
       </c>
       <c r="H15" s="18" t="inlineStr">
         <is>
-          <t>T-System H0202</t>
+          <t>G-TOPAS H0202</t>
         </is>
       </c>
       <c r="I15" s="18" t="inlineStr">
         <is>
-          <t>Supplier System TB_R_H0202</t>
+          <t>NSP TB_R_H0202</t>
         </is>
       </c>
       <c r="J15" s="22" t="inlineStr">
@@ -1956,12 +1956,12 @@
       </c>
       <c r="H16" s="24" t="inlineStr">
         <is>
-          <t>T-System H0253</t>
+          <t>G-TOPAS H0253</t>
         </is>
       </c>
       <c r="I16" s="24" t="inlineStr">
         <is>
-          <t>Supplier System TB_R_H0253_ORDER_CONTROL_PRE</t>
+          <t>NSP TB_R_H0253_ORDER_CONTROL_PRE</t>
         </is>
       </c>
       <c r="J16" s="25" t="inlineStr">
@@ -2013,12 +2013,12 @@
       </c>
       <c r="H17" s="18" t="inlineStr">
         <is>
-          <t>T-System H0125</t>
+          <t>G-TOPAS H0125</t>
         </is>
       </c>
       <c r="I17" s="18" t="inlineStr">
         <is>
-          <t>Supplier System TB_M_H0125_DESTINATION</t>
+          <t>NSP TB_M_H0125_DESTINATION</t>
         </is>
       </c>
       <c r="J17" s="22" t="inlineStr">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>Tim Supplier System / IT (DBA)</t>
+          <t>Tim NSP / IT (DBA)</t>
         </is>
       </c>
       <c r="G13" s="18" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>Tim Supplier System / IT</t>
+          <t>Tim NSP / IT</t>
         </is>
       </c>
       <c r="G14" s="18" t="inlineStr">
@@ -2696,7 +2696,7 @@
       </c>
       <c r="C20" s="18" t="inlineStr">
         <is>
-          <t>Tambah kolom HOLD_FLAG / PO_MAPPED_FLAG di H0253 Supplier System, dipertahankan saat sync X10 (sudah diputuskan)</t>
+          <t>Tambah kolom HOLD_FLAG / PO_MAPPED_FLAG di H0253 NSP, dipertahankan saat sync X10 (sudah diputuskan)</t>
         </is>
       </c>
       <c r="D20" s="18" t="inlineStr">
@@ -2711,7 +2711,7 @@
       </c>
       <c r="F20" s="18" t="inlineStr">
         <is>
-          <t>Tim Supplier System / IT</t>
+          <t>Tim NSP / IT</t>
         </is>
       </c>
       <c r="G20" s="18" t="inlineStr">
@@ -3024,12 +3024,12 @@
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>Jadwal scheduler Supplier System untuk X9, X10, X11 dan perlu auto retry seperti X6 / X7?</t>
+          <t>Jadwal scheduler NSP untuk X9, X10, X11 dan perlu auto retry seperti X6 / X7?</t>
         </is>
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Setelah data T-System tersedia; auto retry 3x.</t>
+          <t>Setelah data G-TOPAS tersedia; auto retry 3x.</t>
         </is>
       </c>
       <c r="G8" s="18" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>Shared folder Supplier System; retensi 12 bulan.</t>
+          <t>Shared folder NSP; retensi 12 bulan.</t>
         </is>
       </c>
       <c r="G19" s="18" t="inlineStr">
@@ -3687,7 +3687,7 @@
     <row r="8" ht="9" customHeight="1">
       <c r="B8" s="34" t="inlineStr">
         <is>
-          <t>T-System /
+          <t>G-TOPAS /
 DB Surrounding</t>
         </is>
       </c>
@@ -3936,7 +3936,7 @@
     <row r="13" ht="9" customHeight="1">
       <c r="B13" s="45" t="inlineStr">
         <is>
-          <t>Supplier System Batch
+          <t>NSP Batch
 (System)</t>
         </is>
       </c>
@@ -4002,7 +4002,7 @@
               <sz val="9"/>
             </rPr>
             <t>Replicate data
-to Supplier System</t>
+to NSP</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
Rename G-TOPAS / GTOPAS to G-System in all documents
Specs, md, UISS (v1 and v2), BPF, ERD, DB Structure, executive overview and
prototype data. File names follow (XD06 ...ToGSystem, gsystem_structure.json,
XD_CDMASTER_GSYSTEM_ file). Physical column TOPAS_ORDER_TYPE is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/exec/Crossdock_Executive_Overview.xlsx
+++ b/deliverables/exec/Crossdock_Executive_Overview.xlsx
@@ -1195,7 +1195,7 @@
     <row r="24" ht="30" customHeight="1">
       <c r="B24" s="19" t="inlineStr">
         <is>
-          <t>✔  Struktur tabel H0202 / H0253 / H0125 dari I/F layout G-TOPAS, termasuk SERIAL_NO</t>
+          <t>✔  Struktur tabel H0202 / H0253 / H0125 dari I/F layout G-System, termasuk SERIAL_NO</t>
         </is>
       </c>
       <c r="H24" s="19" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="H15" s="18" t="inlineStr">
         <is>
-          <t>G-TOPAS H0202</t>
+          <t>G-System H0202</t>
         </is>
       </c>
       <c r="I15" s="18" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="H16" s="24" t="inlineStr">
         <is>
-          <t>G-TOPAS H0253</t>
+          <t>G-System H0253</t>
         </is>
       </c>
       <c r="I16" s="24" t="inlineStr">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="H17" s="18" t="inlineStr">
         <is>
-          <t>G-TOPAS H0125</t>
+          <t>G-System H0125</t>
         </is>
       </c>
       <c r="I17" s="18" t="inlineStr">
@@ -3029,7 +3029,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Setelah data G-TOPAS tersedia; auto retry 3x.</t>
+          <t>Setelah data G-System tersedia; auto retry 3x.</t>
         </is>
       </c>
       <c r="G8" s="18" t="inlineStr">
@@ -3687,7 +3687,7 @@
     <row r="8" ht="9" customHeight="1">
       <c r="B8" s="34" t="inlineStr">
         <is>
-          <t>G-TOPAS /
+          <t>G-System /
 DB Surrounding</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Rename G-System to GTOPAS in documents; web and simulation use G-System
- UISS XD01-XD15 (XD06 file renamed ...ToGTOPAS), first-version UISS X9-X12, md, BPF, ERD, DB Structure, exec overview and UR summary use GTOPAS / NSP
- Prototype web: remaining T-System texts renamed to G-System; BPF page Document names = GTOPAS / NSP
- simulasi_asn_rev.xlsx keeps G-System

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/exec/Crossdock_Executive_Overview.xlsx
+++ b/deliverables/exec/Crossdock_Executive_Overview.xlsx
@@ -1195,7 +1195,7 @@
     <row r="24" ht="30" customHeight="1">
       <c r="B24" s="19" t="inlineStr">
         <is>
-          <t>✔  Struktur tabel H0202 / H0253 / H0125 dari I/F layout G-System, termasuk SERIAL_NO</t>
+          <t>✔  Struktur tabel H0202 / H0253 / H0125 dari I/F layout GTOPAS, termasuk SERIAL_NO</t>
         </is>
       </c>
       <c r="H24" s="19" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="H15" s="18" t="inlineStr">
         <is>
-          <t>G-System H0202</t>
+          <t>GTOPAS H0202</t>
         </is>
       </c>
       <c r="I15" s="18" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="H16" s="24" t="inlineStr">
         <is>
-          <t>G-System H0253</t>
+          <t>GTOPAS H0253</t>
         </is>
       </c>
       <c r="I16" s="24" t="inlineStr">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="H17" s="18" t="inlineStr">
         <is>
-          <t>G-System H0125</t>
+          <t>GTOPAS H0125</t>
         </is>
       </c>
       <c r="I17" s="18" t="inlineStr">
@@ -3029,7 +3029,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Setelah data G-System tersedia; auto retry 3x.</t>
+          <t>Setelah data GTOPAS tersedia; auto retry 3x.</t>
         </is>
       </c>
       <c r="G8" s="18" t="inlineStr">
@@ -3687,7 +3687,7 @@
     <row r="8" ht="9" customHeight="1">
       <c r="B8" s="34" t="inlineStr">
         <is>
-          <t>G-System /
+          <t>GTOPAS /
 DB Surrounding</t>
         </is>
       </c>

</xml_diff>